<commit_message>
fix(export): match the original management workbook layout
Restore original formatting below row 40, name style and order per sheet,
zero rows for unpaid cutoffs, journal entries, and the voucher header,
account names and codes. Notes move out of the print area; signatories
print by name only and no signature pictures are added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/payroll/management-template.xlsx
+++ b/resources/payroll/management-template.xlsx
@@ -3545,99 +3545,34 @@
       <c r="N39" s="37"/>
       <c r="T39" s="48"/>
     </row>
-    <row r="40" spans="1:38" ns2:dyDescent="0.25" ht="35" customHeight="1">
+    <row r="40" spans="1:38" ns2:dyDescent="0.25">
       <c r="T40" s="21"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="34"/>
-      <c r="F40" s="34"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="34"/>
-      <c r="J40" s="34"/>
-      <c r="K40" s="34"/>
-      <c r="L40" s="34"/>
-      <c r="M40" s="34"/>
-      <c r="N40" s="34"/>
-      <c r="O40" s="34"/>
-    </row>
-    <row r="41" ht="35" customHeight="1">
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="34"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="34"/>
-      <c r="J41" s="34"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="34"/>
-      <c r="M41" s="34"/>
-      <c r="N41" s="34"/>
-      <c r="O41" s="34"/>
-    </row>
-    <row r="42" spans="1:38" ns2:dyDescent="0.25" ht="35" customHeight="1">
+    </row>
+    <row r="41"/>
+    <row r="42" spans="1:38" ns2:dyDescent="0.25">
       <c r="AB42" s="5"/>
       <c r="AC42" s="5"/>
       <c r="AG42" s="5"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="11"/>
-      <c r="O42" s="11"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="34"/>
-      <c r="J43" s="34"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="34"/>
-      <c r="M43" s="34"/>
-      <c r="N43" s="34"/>
-      <c r="O43" s="34"/>
-    </row>
-    <row r="44" spans="1:38" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="L44" s="34"/>
+    </row>
+    <row r="43"/>
+    <row r="44" spans="1:38" ns2:dyDescent="0.25">
+      <c r="B44" s="39"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="L44" s="7"/>
       <c r="AC44" s="5"/>
-      <c r="C44" s="14"/>
-      <c r="I44" s="34"/>
-      <c r="J44" s="34"/>
-      <c r="K44" s="34"/>
-      <c r="M44" s="34"/>
-      <c r="N44" s="34"/>
-      <c r="O44" s="34"/>
-    </row>
-    <row r="45" spans="1:38" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="34"/>
-      <c r="F45" s="34"/>
-      <c r="G45" s="34"/>
-      <c r="H45" s="34"/>
-      <c r="L45" s="34"/>
+    </row>
+    <row r="45" spans="1:38" ns2:dyDescent="0.25">
+      <c r="B45" s="10"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="L45" s="112"/>
       <c r="AC45" s="6"/>
       <c r="AD45" s="6"/>
       <c r="AE45" s="6"/>
@@ -3645,15 +3580,8 @@
       <c r="AG45" s="52"/>
       <c r="AH45" s="50"/>
       <c r="AI45" s="50"/>
-      <c r="C45" s="14"/>
-      <c r="I45" s="34"/>
-      <c r="J45" s="34"/>
-      <c r="K45" s="34"/>
-      <c r="M45" s="34"/>
-      <c r="N45" s="34"/>
-      <c r="O45" s="34"/>
-    </row>
-    <row r="46" spans="1:38" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="46" spans="1:38" ns2:dyDescent="0.25">
       <c r="AC46" s="5"/>
       <c r="AD46" s="5"/>
       <c r="AE46" s="5"/>
@@ -3663,203 +3591,23 @@
       <c r="AI46" s="5"/>
       <c r="AJ46" s="5"/>
       <c r="AK46" s="5"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="34"/>
-      <c r="I46" s="34"/>
-      <c r="J46" s="34"/>
-      <c r="K46" s="34"/>
-      <c r="L46" s="34"/>
-      <c r="M46" s="34"/>
-      <c r="N46" s="34"/>
-      <c r="O46" s="34"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="34"/>
-      <c r="F47" s="34"/>
-      <c r="G47" s="34"/>
-      <c r="H47" s="34"/>
-      <c r="I47" s="34"/>
-      <c r="J47" s="34"/>
-      <c r="K47" s="34"/>
-      <c r="L47" s="34"/>
-      <c r="M47" s="34"/>
-      <c r="N47" s="34"/>
-      <c r="O47" s="34"/>
-    </row>
-    <row r="48" spans="1:38" ht="20" customHeight="1" ns2:dyDescent="0.25">
+    </row>
+    <row r="47"/>
+    <row ht="15.6" customHeight="1" r="48" spans="1:38" ns2:dyDescent="0.25">
       <c r="AL48" s="38"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="34"/>
-      <c r="F48" s="34"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="34"/>
-      <c r="I48" s="34"/>
-      <c r="J48" s="34"/>
-      <c r="K48" s="34"/>
-      <c r="L48" s="34"/>
-      <c r="M48" s="34"/>
-      <c r="N48" s="34"/>
-      <c r="O48" s="34"/>
-    </row>
-    <row r="49" spans="28:47" ht="20" customHeight="1" ns2:dyDescent="0.25">
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="49" spans="28:47" ns2:dyDescent="0.25">
       <c r="AL49" s="38"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="34"/>
-      <c r="F49" s="34"/>
-      <c r="G49" s="34"/>
-      <c r="H49" s="34"/>
-      <c r="I49" s="34"/>
-      <c r="J49" s="34"/>
-      <c r="K49" s="34"/>
-      <c r="L49" s="34"/>
-      <c r="M49" s="34"/>
-      <c r="N49" s="34"/>
-      <c r="O49" s="34"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="34"/>
-      <c r="F50" s="34"/>
-      <c r="G50" s="34"/>
-      <c r="H50" s="34"/>
-      <c r="I50" s="34"/>
-      <c r="J50" s="34"/>
-      <c r="K50" s="34"/>
-      <c r="L50" s="34"/>
-      <c r="M50" s="34"/>
-      <c r="N50" s="34"/>
-      <c r="O50" s="34"/>
-    </row>
-    <row r="51" spans="28:47" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="34"/>
-      <c r="F51" s="34"/>
-      <c r="G51" s="34"/>
-      <c r="H51" s="34"/>
-      <c r="I51" s="34"/>
-      <c r="J51" s="34"/>
-      <c r="K51" s="34"/>
-      <c r="L51" s="34"/>
-      <c r="M51" s="34"/>
-      <c r="N51" s="34"/>
-      <c r="O51" s="34"/>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="34"/>
-      <c r="F52" s="34"/>
-      <c r="G52" s="34"/>
-      <c r="H52" s="34"/>
-      <c r="I52" s="34"/>
-      <c r="J52" s="34"/>
-      <c r="K52" s="34"/>
-      <c r="L52" s="34"/>
-      <c r="M52" s="34"/>
-      <c r="N52" s="34"/>
-      <c r="O52" s="34"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="34"/>
-      <c r="F53" s="34"/>
-      <c r="G53" s="34"/>
-      <c r="H53" s="34"/>
-      <c r="I53" s="34"/>
-      <c r="J53" s="34"/>
-      <c r="K53" s="34"/>
-      <c r="L53" s="34"/>
-      <c r="M53" s="34"/>
-      <c r="N53" s="34"/>
-      <c r="O53" s="34"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="34"/>
-      <c r="F54" s="34"/>
-      <c r="G54" s="34"/>
-      <c r="H54" s="34"/>
-      <c r="I54" s="34"/>
-      <c r="J54" s="34"/>
-      <c r="K54" s="34"/>
-      <c r="L54" s="34"/>
-      <c r="M54" s="34"/>
-      <c r="N54" s="34"/>
-      <c r="O54" s="34"/>
-    </row>
-    <row r="55" spans="28:47" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="AL55"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="34"/>
-      <c r="F55" s="34"/>
-      <c r="G55" s="34"/>
-      <c r="H55" s="34"/>
-      <c r="I55" s="34"/>
-      <c r="J55" s="34"/>
-      <c r="K55" s="34"/>
-      <c r="L55" s="34"/>
-      <c r="M55" s="34"/>
-      <c r="N55" s="34"/>
-      <c r="O55" s="34"/>
-    </row>
-    <row r="56" spans="28:47" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="AL56"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="34"/>
-      <c r="F56" s="34"/>
-      <c r="G56" s="34"/>
-      <c r="H56" s="34"/>
-      <c r="I56" s="34"/>
-      <c r="J56" s="34"/>
-      <c r="K56" s="34"/>
-      <c r="L56" s="34"/>
-      <c r="M56" s="34"/>
-      <c r="N56" s="34"/>
-      <c r="O56" s="34"/>
-    </row>
-    <row r="57" spans="28:47" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="AL57"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="34"/>
-      <c r="F57" s="34"/>
-      <c r="G57" s="34"/>
-      <c r="H57" s="34"/>
-      <c r="I57" s="34"/>
-      <c r="J57" s="34"/>
-      <c r="K57" s="34"/>
-      <c r="L57" s="34"/>
-      <c r="M57" s="34"/>
-      <c r="N57" s="34"/>
-      <c r="O57" s="34"/>
-    </row>
-    <row r="58" spans="28:47" ht="20" customHeight="1" ns2:dyDescent="0.35">
+    </row>
+    <row r="50"/>
+    <row ht="16.149999999999999" customHeight="1" r="51" spans="28:47" ns2:dyDescent="0.25"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55" spans="28:47" ns2:dyDescent="0.25"/>
+    <row r="56" spans="28:47" ns2:dyDescent="0.25"/>
+    <row ht="15" customHeight="1" r="57" spans="28:47" ns2:dyDescent="0.25"/>
+    <row ht="16.899999999999999" customHeight="1" r="58" spans="28:47" ns2:dyDescent="0.35">
       <c r="AB58" s="53"/>
       <c r="AC58" s="54"/>
       <c r="AD58" s="54"/>
@@ -3870,57 +3618,12 @@
       <c r="AI58" s="54"/>
       <c r="AJ58" s="54"/>
       <c r="AK58" s="54"/>
-      <c r="AL58"/>
       <c r="AO58" s="53"/>
       <c r="AP58" s="52"/>
       <c r="AQ58" s="55"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="34"/>
-      <c r="F58" s="34"/>
-      <c r="G58" s="34"/>
-      <c r="H58" s="34"/>
-      <c r="I58" s="34"/>
-      <c r="J58" s="34"/>
-      <c r="K58" s="34"/>
-      <c r="L58" s="34"/>
-      <c r="M58" s="34"/>
-      <c r="N58" s="34"/>
-      <c r="O58" s="34"/>
-    </row>
-    <row r="59" spans="28:47" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="34"/>
-      <c r="F59" s="34"/>
-      <c r="G59" s="34"/>
-      <c r="H59" s="34"/>
-      <c r="I59" s="34"/>
-      <c r="J59" s="34"/>
-      <c r="K59" s="34"/>
-      <c r="L59" s="34"/>
-      <c r="M59" s="34"/>
-      <c r="N59" s="34"/>
-      <c r="O59" s="34"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="34"/>
-      <c r="F60" s="34"/>
-      <c r="G60" s="34"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="34"/>
-      <c r="J60" s="34"/>
-      <c r="K60" s="34"/>
-      <c r="L60" s="34"/>
-      <c r="M60" s="34"/>
-      <c r="N60" s="34"/>
-      <c r="O60" s="34"/>
-    </row>
+    </row>
+    <row ht="31.9" customHeight="1" r="59" spans="28:47" ns2:dyDescent="0.25"/>
+    <row r="60"/>
     <row r="61" spans="28:47" ns2:dyDescent="0.25">
       <c r="AS61" s="21"/>
       <c r="AT61" s="21"/>
@@ -3965,7 +3668,7 @@
       <c r="AO72" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="20">
     <mergeCell ref="B8:M8"/>
     <mergeCell ref="O8:Y8"/>
     <mergeCell ref="AB8:AK9"/>
@@ -3986,8 +3689,6 @@
     <mergeCell ref="B33:N33"/>
     <mergeCell ref="K19:L19"/>
     <mergeCell ref="B14:J14"/>
-    <mergeCell ref="B40:O40"/>
-    <mergeCell ref="B41:O41"/>
   </mergeCells>
   <conditionalFormatting sqref="AB11 AB13">
     <cfRule type="duplicateValues" dxfId="5" priority="40"/>
@@ -5328,195 +5029,184 @@
       <c r="S39" s="21"/>
       <c r="T39" s="48"/>
     </row>
-    <row r="40" spans="1:34" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="N40" s="17"/>
+    <row r="40" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B40" s="151"/>
+      <c r="C40" s="151"/>
+      <c r="D40" s="151"/>
+      <c r="E40" s="151"/>
+      <c r="F40" s="151"/>
+      <c r="G40" s="151"/>
+      <c r="H40" s="151"/>
+      <c r="I40" s="151"/>
+      <c r="J40" s="151"/>
+      <c r="K40" s="151"/>
+      <c r="L40" s="151"/>
+      <c r="M40" s="151"/>
+      <c r="N40" s="151"/>
       <c r="T40" s="48"/>
-      <c r="O40" s="17"/>
-    </row>
-    <row r="41" spans="1:34" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
+    </row>
+    <row r="41" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B41" s="151"/>
+      <c r="C41" s="151"/>
+      <c r="D41" s="151"/>
+      <c r="E41" s="151"/>
+      <c r="F41" s="151"/>
+      <c r="G41" s="151"/>
+      <c r="H41" s="151"/>
+      <c r="I41" s="151"/>
+      <c r="J41" s="151"/>
+      <c r="K41" s="151"/>
+      <c r="L41" s="151"/>
+      <c r="M41" s="151"/>
+      <c r="N41" s="151"/>
       <c r="T41" s="48"/>
-      <c r="O41" s="17"/>
-    </row>
-    <row r="42" spans="1:34" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="11"/>
+    </row>
+    <row r="42" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B42" s="39"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="113"/>
+      <c r="E42" s="113"/>
+      <c r="F42" s="113"/>
+      <c r="G42" s="113"/>
+      <c r="H42" s="113"/>
+      <c r="I42" s="113"/>
+      <c r="J42" s="113"/>
+      <c r="K42" s="113"/>
+      <c r="L42" s="113"/>
+      <c r="M42" s="113"/>
+      <c r="N42" s="113"/>
       <c r="T42" s="5"/>
       <c r="AD42" s="5"/>
       <c r="AG42" s="5"/>
       <c r="AH42" s="50"/>
-      <c r="O42" s="11"/>
-    </row>
-    <row r="43" spans="1:34" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
+    </row>
+    <row r="43" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B43" s="53"/>
+      <c r="C43" s="114"/>
+      <c r="D43" s="115"/>
+      <c r="E43" s="116"/>
+      <c r="F43" s="116"/>
+      <c r="G43" s="123"/>
+      <c r="H43" s="116"/>
+      <c r="I43" s="116"/>
+      <c r="J43" s="116"/>
+      <c r="K43" s="116"/>
+      <c r="L43" s="124"/>
+      <c r="M43" s="124"/>
+      <c r="N43" s="124"/>
       <c r="T43" s="48"/>
-      <c r="O43" s="17"/>
-    </row>
-    <row r="44" spans="1:34" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
+    </row>
+    <row r="44" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B44" s="53"/>
+      <c r="C44" s="114"/>
+      <c r="D44" s="115"/>
+      <c r="E44" s="116"/>
+      <c r="F44" s="116"/>
+      <c r="G44" s="123"/>
+      <c r="H44" s="116"/>
+      <c r="I44" s="116"/>
+      <c r="J44" s="116"/>
+      <c r="K44" s="116"/>
+      <c r="L44" s="124"/>
+      <c r="M44" s="124"/>
+      <c r="N44" s="124"/>
       <c r="T44" s="21"/>
-      <c r="O44" s="17"/>
-    </row>
-    <row r="45" spans="1:34" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
-    </row>
-    <row r="46" spans="1:34" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
-      <c r="N46" s="17"/>
+    </row>
+    <row r="45" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B45" s="53"/>
+      <c r="C45" s="114"/>
+      <c r="D45" s="115"/>
+      <c r="E45" s="116"/>
+      <c r="F45" s="116"/>
+      <c r="G45" s="123"/>
+      <c r="H45" s="116"/>
+      <c r="I45" s="116"/>
+      <c r="J45" s="116"/>
+      <c r="K45" s="116"/>
+      <c r="L45" s="124"/>
+      <c r="M45" s="124"/>
+      <c r="N45" s="124"/>
+    </row>
+    <row r="46" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B46" s="53"/>
+      <c r="C46" s="114"/>
+      <c r="D46" s="115"/>
+      <c r="E46" s="116"/>
+      <c r="F46" s="116"/>
+      <c r="G46" s="123"/>
+      <c r="H46" s="116"/>
+      <c r="I46" s="116"/>
+      <c r="J46" s="116"/>
+      <c r="K46" s="116"/>
+      <c r="L46" s="124"/>
+      <c r="M46" s="124"/>
+      <c r="N46" s="124"/>
       <c r="AC46" s="5"/>
       <c r="AD46" s="5"/>
       <c r="AH46" s="5"/>
-      <c r="O46" s="17"/>
-    </row>
-    <row r="47" spans="1:34" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
-    </row>
-    <row r="48" spans="1:34" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="17"/>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="17"/>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
-    </row>
-    <row r="49" spans="2:44" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
-    </row>
-    <row r="50" spans="2:44" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="17"/>
-      <c r="L50" s="17"/>
-      <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
+    </row>
+    <row r="47" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B47" s="53"/>
+      <c r="C47" s="114"/>
+      <c r="D47" s="115"/>
+      <c r="E47" s="116"/>
+      <c r="F47" s="116"/>
+      <c r="G47" s="123"/>
+      <c r="H47" s="116"/>
+      <c r="I47" s="116"/>
+      <c r="J47" s="116"/>
+      <c r="K47" s="116"/>
+      <c r="L47" s="124"/>
+      <c r="M47" s="124"/>
+      <c r="N47" s="124"/>
+    </row>
+    <row r="48" spans="1:34" ns2:dyDescent="0.25">
+      <c r="B48" s="53"/>
+      <c r="C48" s="114"/>
+      <c r="D48" s="115"/>
+      <c r="E48" s="116"/>
+      <c r="F48" s="116"/>
+      <c r="G48" s="123"/>
+      <c r="H48" s="116"/>
+      <c r="I48" s="116"/>
+      <c r="J48" s="116"/>
+      <c r="K48" s="116"/>
+      <c r="L48" s="124"/>
+      <c r="M48" s="124"/>
+      <c r="N48" s="124"/>
+    </row>
+    <row r="49" spans="2:44" ns2:dyDescent="0.25">
+      <c r="B49" s="53"/>
+      <c r="C49" s="114"/>
+      <c r="D49" s="115"/>
+      <c r="E49" s="116"/>
+      <c r="F49" s="116"/>
+      <c r="G49" s="123"/>
+      <c r="H49" s="116"/>
+      <c r="I49" s="116"/>
+      <c r="J49" s="116"/>
+      <c r="K49" s="116"/>
+      <c r="L49" s="124"/>
+      <c r="M49" s="124"/>
+      <c r="N49" s="124"/>
+    </row>
+    <row r="50" spans="2:44" ns2:dyDescent="0.25">
+      <c r="B50" s="149"/>
+      <c r="C50" s="149"/>
+      <c r="D50" s="149"/>
+      <c r="E50" s="149"/>
+      <c r="F50" s="149"/>
+      <c r="G50" s="149"/>
+      <c r="H50" s="149"/>
+      <c r="I50" s="149"/>
+      <c r="J50" s="149"/>
+      <c r="K50" s="149"/>
+      <c r="L50" s="36"/>
+      <c r="M50" s="36"/>
+      <c r="N50" s="36"/>
       <c r="AD50" s="5"/>
-      <c r="O50" s="17"/>
-    </row>
-    <row r="51" spans="2:44" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="51" spans="2:44" ns2:dyDescent="0.25">
       <c r="AD51" s="6"/>
       <c r="AE51" s="6"/>
       <c r="AF51" s="6"/>
@@ -5524,22 +5214,8 @@
       <c r="AH51" s="52"/>
       <c r="AI51" s="50"/>
       <c r="AJ51" s="50"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="17"/>
-      <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
-    </row>
-    <row r="52" spans="2:44" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="52" spans="2:44" ns2:dyDescent="0.25">
       <c r="AD52" s="5"/>
       <c r="AE52" s="5"/>
       <c r="AF52" s="5"/>
@@ -5549,161 +5225,40 @@
       <c r="AJ52" s="5"/>
       <c r="AK52" s="5"/>
       <c r="AL52" s="5"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="17"/>
-      <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
-    </row>
-    <row r="54" spans="2:44" ht="20" customHeight="1" ns2:dyDescent="0.25">
+    </row>
+    <row r="53"/>
+    <row ht="15.6" customHeight="1" r="54" spans="2:44" ns2:dyDescent="0.25">
       <c r="AM54" s="38"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
-      <c r="K54" s="17"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
-    </row>
-    <row r="55" spans="2:44" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
-      <c r="G55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="55" spans="2:44" ns2:dyDescent="0.25">
+      <c r="B55" s="39"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+      <c r="L55" s="8"/>
+      <c r="M55" s="8"/>
       <c r="AM55" s="38"/>
-      <c r="C55" s="14"/>
-      <c r="I55" s="17"/>
-      <c r="J55" s="17"/>
-      <c r="K55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
-    </row>
-    <row r="56" spans="2:44" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="17"/>
-      <c r="F56" s="17"/>
-      <c r="G56" s="17"/>
-      <c r="H56" s="17"/>
-      <c r="L56" s="17"/>
-      <c r="M56" s="17"/>
-      <c r="C56" s="14"/>
-      <c r="I56" s="17"/>
-      <c r="J56" s="17"/>
-      <c r="K56" s="17"/>
-      <c r="N56" s="17"/>
-      <c r="O56" s="17"/>
-    </row>
-    <row r="57" spans="2:44" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="17"/>
-      <c r="I58" s="17"/>
-      <c r="J58" s="17"/>
-      <c r="K58" s="17"/>
-      <c r="L58" s="17"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
-      <c r="O58" s="17"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
-      <c r="M59" s="17"/>
-      <c r="N59" s="17"/>
-      <c r="O59" s="17"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-      <c r="H60" s="17"/>
-      <c r="I60" s="17"/>
-      <c r="J60" s="17"/>
-      <c r="K60" s="17"/>
-      <c r="L60" s="17"/>
-      <c r="M60" s="17"/>
-      <c r="N60" s="17"/>
-      <c r="O60" s="17"/>
-    </row>
-    <row r="61" spans="2:44" ns2:dyDescent="0.25">
-      <c r="AM61"/>
-    </row>
-    <row r="62" spans="2:44" ns2:dyDescent="0.25">
-      <c r="AM62"/>
-    </row>
-    <row r="63" spans="2:44" ht="15" customHeight="1" ns2:dyDescent="0.25">
-      <c r="AM63"/>
-    </row>
-    <row r="64" spans="2:44" ht="16.899999999999999" customHeight="1" ns2:dyDescent="0.35">
+    </row>
+    <row r="56" spans="2:44" ns2:dyDescent="0.25">
+      <c r="B56" s="10"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="L56" s="153"/>
+      <c r="M56" s="153"/>
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="57" spans="2:44" ns2:dyDescent="0.25"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61" spans="2:44" ns2:dyDescent="0.25"/>
+    <row r="62" spans="2:44" ns2:dyDescent="0.25"/>
+    <row ht="15" customHeight="1" r="63" spans="2:44" ns2:dyDescent="0.25"/>
+    <row ht="16.899999999999999" customHeight="1" r="64" spans="2:44" ns2:dyDescent="0.35">
       <c r="AC64" s="53"/>
       <c r="AD64" s="54"/>
       <c r="AE64" s="54"/>
@@ -5714,12 +5269,11 @@
       <c r="AJ64" s="54"/>
       <c r="AK64" s="54"/>
       <c r="AL64" s="54"/>
-      <c r="AM64"/>
       <c r="AP64" s="53"/>
       <c r="AQ64" s="52"/>
       <c r="AR64" s="55"/>
     </row>
-    <row r="65" spans="42:48" ht="31.9" customHeight="1" ns2:dyDescent="0.25"/>
+    <row ht="31.9" customHeight="1" r="65" spans="42:48" ns2:dyDescent="0.25"/>
     <row r="67" spans="42:48" ns2:dyDescent="0.25">
       <c r="AT67" s="21"/>
       <c r="AU67" s="21"/>
@@ -5764,7 +5318,7 @@
       <c r="AP78" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="21">
     <mergeCell ref="B50:K50"/>
     <mergeCell ref="L56:M56"/>
     <mergeCell ref="K19:L19"/>
@@ -5786,8 +5340,6 @@
     <mergeCell ref="AC8:AL9"/>
     <mergeCell ref="B9:M9"/>
     <mergeCell ref="O9:Z9"/>
-    <mergeCell ref="B40:O40"/>
-    <mergeCell ref="B41:O41"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7014,195 +6566,151 @@
       <c r="P39" s="21"/>
       <c r="Q39" s="48"/>
     </row>
-    <row r="40" spans="1:29" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
+    <row r="40" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B40" s="151"/>
+      <c r="C40" s="151"/>
+      <c r="D40" s="151"/>
+      <c r="E40" s="151"/>
+      <c r="F40" s="151"/>
+      <c r="G40" s="151"/>
+      <c r="H40" s="151"/>
+      <c r="I40" s="151"/>
+      <c r="J40" s="151"/>
+      <c r="K40" s="151"/>
       <c r="Q40" s="48"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="N40" s="17"/>
-      <c r="O40" s="17"/>
-    </row>
-    <row r="41" spans="1:29" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
+    </row>
+    <row r="41" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B41" s="151"/>
+      <c r="C41" s="151"/>
+      <c r="D41" s="151"/>
+      <c r="E41" s="151"/>
+      <c r="F41" s="151"/>
+      <c r="G41" s="151"/>
+      <c r="H41" s="151"/>
+      <c r="I41" s="151"/>
+      <c r="J41" s="151"/>
+      <c r="K41" s="151"/>
       <c r="Q41" s="48"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
-    </row>
-    <row r="42" spans="1:29" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11"/>
+    </row>
+    <row r="42" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B42" s="39"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="113"/>
+      <c r="E42" s="113"/>
+      <c r="F42" s="113"/>
+      <c r="G42" s="113"/>
+      <c r="H42" s="113"/>
+      <c r="I42" s="113"/>
+      <c r="J42" s="113"/>
+      <c r="K42" s="113"/>
       <c r="Q42" s="5"/>
       <c r="Y42" s="5"/>
       <c r="AB42" s="5"/>
       <c r="AC42" s="50"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="11"/>
-      <c r="O42" s="11"/>
-    </row>
-    <row r="43" spans="1:29" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
+    </row>
+    <row r="43" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B43" s="53"/>
+      <c r="C43" s="114"/>
+      <c r="D43" s="115"/>
+      <c r="E43" s="116"/>
+      <c r="F43" s="123"/>
+      <c r="G43" s="116"/>
+      <c r="H43" s="124"/>
+      <c r="I43" s="124"/>
+      <c r="J43" s="124"/>
+      <c r="K43" s="124"/>
       <c r="Q43" s="48"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
-      <c r="O43" s="17"/>
-    </row>
-    <row r="44" spans="1:29" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
+    </row>
+    <row r="44" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B44" s="53"/>
+      <c r="C44" s="114"/>
+      <c r="D44" s="115"/>
+      <c r="E44" s="116"/>
+      <c r="F44" s="123"/>
+      <c r="G44" s="116"/>
+      <c r="H44" s="124"/>
+      <c r="I44" s="124"/>
+      <c r="J44" s="124"/>
+      <c r="K44" s="124"/>
       <c r="Q44" s="21"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
-      <c r="O44" s="17"/>
-    </row>
-    <row r="45" spans="1:29" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
-    </row>
-    <row r="46" spans="1:29" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
+    </row>
+    <row r="45" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B45" s="53"/>
+      <c r="C45" s="114"/>
+      <c r="D45" s="115"/>
+      <c r="E45" s="116"/>
+      <c r="F45" s="123"/>
+      <c r="G45" s="116"/>
+      <c r="H45" s="124"/>
+      <c r="I45" s="124"/>
+      <c r="J45" s="124"/>
+      <c r="K45" s="124"/>
+    </row>
+    <row r="46" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B46" s="53"/>
+      <c r="C46" s="114"/>
+      <c r="D46" s="115"/>
+      <c r="E46" s="116"/>
+      <c r="F46" s="123"/>
+      <c r="G46" s="116"/>
+      <c r="H46" s="124"/>
+      <c r="I46" s="124"/>
+      <c r="J46" s="124"/>
+      <c r="K46" s="124"/>
       <c r="X46" s="5"/>
       <c r="Y46" s="5"/>
       <c r="AC46" s="5"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
-      <c r="N46" s="17"/>
-      <c r="O46" s="17"/>
-    </row>
-    <row r="47" spans="1:29" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
-    </row>
-    <row r="48" spans="1:29" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="17"/>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="17"/>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
-    </row>
-    <row r="49" spans="2:39" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
-    </row>
-    <row r="50" spans="2:39" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="17"/>
+    </row>
+    <row r="47" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B47" s="53"/>
+      <c r="C47" s="114"/>
+      <c r="D47" s="115"/>
+      <c r="E47" s="116"/>
+      <c r="F47" s="123"/>
+      <c r="G47" s="116"/>
+      <c r="H47" s="124"/>
+      <c r="I47" s="124"/>
+      <c r="J47" s="124"/>
+      <c r="K47" s="124"/>
+    </row>
+    <row r="48" spans="1:29" ns2:dyDescent="0.25">
+      <c r="B48" s="53"/>
+      <c r="C48" s="114"/>
+      <c r="D48" s="115"/>
+      <c r="E48" s="116"/>
+      <c r="F48" s="123"/>
+      <c r="G48" s="116"/>
+      <c r="H48" s="124"/>
+      <c r="I48" s="124"/>
+      <c r="J48" s="124"/>
+      <c r="K48" s="124"/>
+    </row>
+    <row r="49" spans="2:39" ns2:dyDescent="0.25">
+      <c r="B49" s="53"/>
+      <c r="C49" s="114"/>
+      <c r="D49" s="115"/>
+      <c r="E49" s="116"/>
+      <c r="F49" s="123"/>
+      <c r="G49" s="116"/>
+      <c r="H49" s="124"/>
+      <c r="I49" s="124"/>
+      <c r="J49" s="124"/>
+      <c r="K49" s="124"/>
+    </row>
+    <row r="50" spans="2:39" ns2:dyDescent="0.25">
+      <c r="B50" s="149"/>
+      <c r="C50" s="149"/>
+      <c r="D50" s="149"/>
+      <c r="E50" s="149"/>
+      <c r="F50" s="149"/>
+      <c r="G50" s="149"/>
+      <c r="H50" s="36"/>
+      <c r="I50" s="36"/>
+      <c r="J50" s="36"/>
+      <c r="K50" s="36"/>
       <c r="Y50" s="5"/>
-      <c r="L50" s="17"/>
-      <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
-      <c r="O50" s="17"/>
-    </row>
-    <row r="51" spans="2:39" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="51" spans="2:39" ns2:dyDescent="0.25">
       <c r="Y51" s="6"/>
       <c r="Z51" s="6"/>
       <c r="AA51" s="6"/>
@@ -7210,22 +6718,8 @@
       <c r="AC51" s="52"/>
       <c r="AD51" s="50"/>
       <c r="AE51" s="50"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="17"/>
-      <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
-    </row>
-    <row r="52" spans="2:39" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="52" spans="2:39" ns2:dyDescent="0.25">
       <c r="Y52" s="5"/>
       <c r="Z52" s="5"/>
       <c r="AA52" s="5"/>
@@ -7235,161 +6729,38 @@
       <c r="AE52" s="5"/>
       <c r="AF52" s="5"/>
       <c r="AG52" s="5"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="17"/>
-      <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
-    </row>
-    <row r="54" spans="2:39" ht="20" customHeight="1" ns2:dyDescent="0.25">
+    </row>
+    <row r="53"/>
+    <row ht="15.6" customHeight="1" r="54" spans="2:39" ns2:dyDescent="0.25">
       <c r="AH54" s="38"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
-      <c r="K54" s="17"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
-    </row>
-    <row r="55" spans="2:39" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
-      <c r="J55" s="17"/>
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="55" spans="2:39" ns2:dyDescent="0.25">
+      <c r="B55" s="39"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="H55" s="8"/>
+      <c r="I55" s="8"/>
+      <c r="J55" s="8"/>
       <c r="AH55" s="38"/>
-      <c r="C55" s="14"/>
-      <c r="G55" s="17"/>
-      <c r="K55" s="17"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
-    </row>
-    <row r="56" spans="2:39" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="17"/>
-      <c r="F56" s="17"/>
-      <c r="H56" s="17"/>
-      <c r="I56" s="17"/>
-      <c r="J56" s="17"/>
-      <c r="C56" s="14"/>
-      <c r="G56" s="17"/>
-      <c r="K56" s="17"/>
-      <c r="L56" s="17"/>
-      <c r="M56" s="17"/>
-      <c r="N56" s="17"/>
-      <c r="O56" s="17"/>
-    </row>
-    <row r="57" spans="2:39" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="17"/>
-      <c r="I58" s="17"/>
-      <c r="J58" s="17"/>
-      <c r="K58" s="17"/>
-      <c r="L58" s="17"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
-      <c r="O58" s="17"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
-      <c r="M59" s="17"/>
-      <c r="N59" s="17"/>
-      <c r="O59" s="17"/>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-      <c r="H60" s="17"/>
-      <c r="I60" s="17"/>
-      <c r="J60" s="17"/>
-      <c r="K60" s="17"/>
-      <c r="L60" s="17"/>
-      <c r="M60" s="17"/>
-      <c r="N60" s="17"/>
-      <c r="O60" s="17"/>
-    </row>
-    <row r="61" spans="2:39" ns2:dyDescent="0.25">
-      <c r="AH61"/>
-    </row>
-    <row r="62" spans="2:39" ns2:dyDescent="0.25">
-      <c r="AH62"/>
-    </row>
-    <row r="63" spans="2:39" ht="15" customHeight="1" ns2:dyDescent="0.25">
-      <c r="AH63"/>
-    </row>
-    <row r="64" spans="2:39" ht="16.899999999999999" customHeight="1" ns2:dyDescent="0.35">
+    </row>
+    <row r="56" spans="2:39" ns2:dyDescent="0.25">
+      <c r="B56" s="10"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="H56" s="153"/>
+      <c r="I56" s="153"/>
+      <c r="J56" s="112"/>
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="57" spans="2:39" ns2:dyDescent="0.25"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61" spans="2:39" ns2:dyDescent="0.25"/>
+    <row r="62" spans="2:39" ns2:dyDescent="0.25"/>
+    <row ht="15" customHeight="1" r="63" spans="2:39" ns2:dyDescent="0.25"/>
+    <row ht="16.899999999999999" customHeight="1" r="64" spans="2:39" ns2:dyDescent="0.35">
       <c r="X64" s="53"/>
       <c r="Y64" s="54"/>
       <c r="Z64" s="54"/>
@@ -7400,12 +6771,11 @@
       <c r="AE64" s="54"/>
       <c r="AF64" s="54"/>
       <c r="AG64" s="54"/>
-      <c r="AH64"/>
       <c r="AK64" s="53"/>
       <c r="AL64" s="52"/>
       <c r="AM64" s="55"/>
     </row>
-    <row r="65" spans="37:43" ht="31.9" customHeight="1" ns2:dyDescent="0.25"/>
+    <row ht="31.9" customHeight="1" r="65" spans="37:43" ns2:dyDescent="0.25"/>
     <row r="67" spans="37:43" ns2:dyDescent="0.25">
       <c r="AO67" s="21"/>
       <c r="AP67" s="21"/>
@@ -7450,7 +6820,7 @@
       <c r="AK78" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="21">
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="X8:AG9"/>
@@ -7472,8 +6842,6 @@
     <mergeCell ref="B32:G32"/>
     <mergeCell ref="B40:K40"/>
     <mergeCell ref="B41:K41"/>
-    <mergeCell ref="B40:O40"/>
-    <mergeCell ref="B41:O41"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8895,128 +8263,97 @@
       </c>
       <c r="R39" s="5"/>
     </row>
-    <row r="40" spans="1:54" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="D40" s="14"/>
-      <c r="N40" s="17"/>
-      <c r="P40" s="1" t="inlineStr">
+    <row r="40" spans="1:54" ns2:dyDescent="0.25">
+      <c r="D40" s="2"/>
+      <c r="N40" s="3"/>
+      <c r="P40" t="inlineStr" s="1">
         <is>
           <t>     SSS Payable - Employer</t>
         </is>
       </c>
       <c r="S40" s="5"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-      <c r="O40" s="17"/>
-    </row>
-    <row r="41" spans="1:54" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="D41" s="14"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="P41" s="1" t="inlineStr">
+    </row>
+    <row r="41" spans="1:54" ns2:dyDescent="0.25">
+      <c r="D41" s="2"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="P41" t="inlineStr" s="1">
         <is>
           <t>     Phil Health Payable - Employer</t>
         </is>
       </c>
       <c r="S41" s="48"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="17"/>
-      <c r="O41" s="17"/>
-    </row>
-    <row r="42" spans="1:54" ns2:dyDescent="0.25" ht="35" customHeight="1">
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="P42" s="1" t="inlineStr">
+    </row>
+    <row r="42" spans="1:54" ns2:dyDescent="0.25">
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="P42" t="inlineStr" s="1">
         <is>
           <t>     PAGIBIG Contribution - Employer</t>
         </is>
       </c>
       <c r="S42" s="21"/>
       <c r="T42" s="48"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="11"/>
-      <c r="O42" s="11"/>
-    </row>
-    <row r="43" spans="1:54" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
+    </row>
+    <row r="43" spans="1:54" ns2:dyDescent="0.25">
+      <c r="B43" s="151"/>
+      <c r="C43" s="151"/>
+      <c r="D43" s="151"/>
+      <c r="E43" s="151"/>
+      <c r="F43" s="151"/>
+      <c r="G43" s="151"/>
+      <c r="H43" s="151"/>
+      <c r="I43" s="151"/>
+      <c r="J43" s="151"/>
+      <c r="K43" s="151"/>
+      <c r="L43" s="151"/>
+      <c r="M43" s="151"/>
+      <c r="N43" s="151"/>
       <c r="T43" s="48"/>
-      <c r="O43" s="17"/>
-    </row>
-    <row r="44" spans="1:54" ht="20" thickBot="1" ns2:dyDescent="0.3" customHeight="1">
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-      <c r="N44" s="17"/>
+    </row>
+    <row ht="16.5" customHeight="1" r="44" spans="1:54" thickBot="1" ns2:dyDescent="0.3">
+      <c r="B44" s="156"/>
+      <c r="C44" s="156"/>
+      <c r="D44" s="156"/>
+      <c r="E44" s="156"/>
+      <c r="F44" s="156"/>
+      <c r="G44" s="156"/>
+      <c r="H44" s="156"/>
+      <c r="I44" s="156"/>
+      <c r="J44" s="156"/>
+      <c r="K44" s="156"/>
+      <c r="L44" s="156"/>
+      <c r="M44" s="156"/>
+      <c r="N44" s="151"/>
       <c r="T44" s="48"/>
-      <c r="O44" s="17"/>
-    </row>
-    <row r="45" spans="1:54" ht="20" thickTop="1" ns2:dyDescent="0.25" customHeight="1">
-      <c r="B45" s="14" t="inlineStr">
+    </row>
+    <row ht="48" customHeight="1" r="45" spans="1:54" thickTop="1" ns2:dyDescent="0.25">
+      <c r="B45" t="inlineStr" s="11">
         <is>
           <t>EMPLOYEE NAME</t>
         </is>
       </c>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17" t="inlineStr">
+      <c r="C45" s="11"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
+      <c r="F45" t="inlineStr" s="12">
         <is>
           <t>OVERTIME PAY</t>
         </is>
       </c>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17" t="inlineStr">
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="12"/>
+      <c r="M45" t="inlineStr" s="13">
         <is>
           <t>NET PAY</t>
         </is>
@@ -9025,161 +8362,141 @@
       <c r="AD45" s="5"/>
       <c r="AG45" s="5"/>
       <c r="AH45" s="50"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
-    </row>
-    <row r="46" spans="1:54" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="46" spans="1:54" ns2:dyDescent="0.25">
       <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="16"/>
       <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
+      <c r="F46" s="120"/>
       <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="17"/>
       <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
-      <c r="M46" s="17"/>
+      <c r="K46" s="18"/>
+      <c r="L46" s="18"/>
+      <c r="M46" s="18"/>
       <c r="T46" s="48"/>
-      <c r="N46" s="17"/>
-      <c r="O46" s="17"/>
-    </row>
-    <row r="47" spans="1:54" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="47" spans="1:54" ns2:dyDescent="0.25">
       <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="16"/>
       <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
+      <c r="F47" s="120"/>
       <c r="G47" s="17"/>
       <c r="H47" s="17"/>
       <c r="I47" s="17"/>
       <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="18"/>
+      <c r="M47" s="18"/>
       <c r="T47" s="21"/>
-      <c r="N47" s="17"/>
-      <c r="O47" s="17"/>
-    </row>
-    <row r="48" spans="1:54" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="48" spans="1:54" ns2:dyDescent="0.25">
       <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="16"/>
       <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
+      <c r="F48" s="120"/>
       <c r="G48" s="17"/>
       <c r="H48" s="17"/>
       <c r="I48" s="17"/>
       <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="17"/>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="17"/>
-    </row>
-    <row r="49" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="18"/>
+    </row>
+    <row r="49" spans="2:40" ns2:dyDescent="0.25">
       <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="16"/>
       <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
+      <c r="F49" s="120"/>
       <c r="G49" s="17"/>
       <c r="H49" s="17"/>
       <c r="I49" s="17"/>
       <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
-    </row>
-    <row r="50" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18"/>
+    </row>
+    <row r="50" spans="2:40" ns2:dyDescent="0.25">
       <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="16"/>
       <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
+      <c r="F50" s="120"/>
       <c r="G50" s="17"/>
       <c r="H50" s="17"/>
       <c r="I50" s="17"/>
       <c r="J50" s="17"/>
-      <c r="K50" s="17"/>
-      <c r="L50" s="17"/>
-      <c r="M50" s="17"/>
-      <c r="N50" s="17"/>
-      <c r="O50" s="17"/>
-    </row>
-    <row r="51" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18"/>
+    </row>
+    <row r="51" spans="2:40" ns2:dyDescent="0.25">
       <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="16"/>
       <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
+      <c r="F51" s="120"/>
       <c r="G51" s="17"/>
       <c r="H51" s="17"/>
       <c r="I51" s="17"/>
       <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="17"/>
-      <c r="O51" s="17"/>
-    </row>
-    <row r="52" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+      <c r="K51" s="18"/>
+      <c r="L51" s="18"/>
+      <c r="M51" s="18"/>
+    </row>
+    <row r="52" spans="2:40" ns2:dyDescent="0.25">
       <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="16"/>
       <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
+      <c r="F52" s="120"/>
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
       <c r="I52" s="17"/>
       <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="17"/>
-      <c r="N52" s="17"/>
-      <c r="O52" s="17"/>
-    </row>
-    <row r="53" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+      <c r="K52" s="18"/>
+      <c r="L52" s="18"/>
+      <c r="M52" s="18"/>
+    </row>
+    <row r="53" spans="2:40" ns2:dyDescent="0.25">
       <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="16"/>
       <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
+      <c r="F53" s="120"/>
       <c r="G53" s="17"/>
       <c r="H53" s="17"/>
       <c r="I53" s="17"/>
       <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
-    </row>
-    <row r="54" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B54" s="14" t="inlineStr">
+      <c r="K53" s="18"/>
+      <c r="L53" s="18"/>
+      <c r="M53" s="18"/>
+    </row>
+    <row r="54" spans="2:40" ns2:dyDescent="0.25">
+      <c r="B54" t="inlineStr" s="149">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
-      <c r="K54" s="17"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
+      <c r="C54" s="149"/>
+      <c r="D54" s="149"/>
+      <c r="E54" s="149"/>
+      <c r="F54" s="149"/>
+      <c r="G54" s="149"/>
+      <c r="H54" s="149"/>
+      <c r="I54" s="149"/>
+      <c r="J54" s="149"/>
+      <c r="K54" s="36"/>
+      <c r="L54" s="36"/>
+      <c r="M54" s="36"/>
       <c r="AD54" s="5"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
-    </row>
-    <row r="55" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="55" spans="2:40" ns2:dyDescent="0.25">
       <c r="AD55" s="6"/>
       <c r="AE55" s="6"/>
       <c r="AF55" s="6"/>
@@ -9188,22 +8505,8 @@
       <c r="AI55" s="50"/>
       <c r="AJ55" s="50"/>
       <c r="AK55" s="50"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
-      <c r="G55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
-      <c r="J55" s="17"/>
-      <c r="K55" s="17"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
-    </row>
-    <row r="56" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
+    </row>
+    <row r="56" spans="2:40" ns2:dyDescent="0.25">
       <c r="AD56" s="5"/>
       <c r="AE56" s="5"/>
       <c r="AF56" s="5"/>
@@ -9214,122 +8517,65 @@
       <c r="AK56" s="5"/>
       <c r="AL56" s="5"/>
       <c r="AM56" s="5"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="17"/>
-      <c r="F56" s="17"/>
-      <c r="G56" s="17"/>
-      <c r="H56" s="17"/>
-      <c r="I56" s="17"/>
-      <c r="J56" s="17"/>
-      <c r="K56" s="17"/>
-      <c r="L56" s="17"/>
-      <c r="M56" s="17"/>
-      <c r="N56" s="17"/>
-      <c r="O56" s="17"/>
-    </row>
-    <row r="57" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B57" s="14" t="inlineStr">
+    </row>
+    <row r="57" spans="2:40" ns2:dyDescent="0.25">
+      <c r="B57" t="inlineStr" s="1">
         <is>
           <t>Prepared by:</t>
         </is>
       </c>
-      <c r="D57" s="14" t="inlineStr">
+      <c r="D57" t="inlineStr" s="1">
         <is>
           <t>Certified Correct:</t>
         </is>
       </c>
-      <c r="K57" s="17" t="inlineStr">
+      <c r="K57" t="inlineStr" s="1">
         <is>
           <t>Approved by:</t>
         </is>
       </c>
-      <c r="C57" s="14"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
-    </row>
-    <row r="58" spans="2:40" ht="20" customHeight="1" ns2:dyDescent="0.25">
+    </row>
+    <row ht="15.6" customHeight="1" r="58" spans="2:40" ns2:dyDescent="0.25">
       <c r="AN58" s="38"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="17"/>
-      <c r="I58" s="17"/>
-      <c r="J58" s="17"/>
-      <c r="K58" s="17"/>
-      <c r="L58" s="17"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="17"/>
-      <c r="O58" s="17"/>
-    </row>
-    <row r="59" spans="2:40" ht="20" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="L59" s="17"/>
-      <c r="M59" s="17"/>
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="59" spans="2:40" ns2:dyDescent="0.25">
+      <c r="B59" s="39"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+      <c r="L59" s="8"/>
+      <c r="M59" s="8"/>
       <c r="AN59" s="38"/>
-      <c r="C59" s="14"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
-      <c r="N59" s="17"/>
-      <c r="O59" s="17"/>
-    </row>
-    <row r="60" spans="2:40" ns2:dyDescent="0.25" ht="20" customHeight="1">
-      <c r="B60" s="14" t="inlineStr">
+    </row>
+    <row r="60" spans="2:40" ns2:dyDescent="0.25">
+      <c r="B60" t="inlineStr" s="10">
         <is>
           <t>PAYROLL OFFICER</t>
         </is>
       </c>
-      <c r="D60" s="14"/>
-      <c r="E60" s="17" t="inlineStr">
+      <c r="D60" s="4"/>
+      <c r="E60" t="inlineStr" s="4">
         <is>
           <t>ACCOUNTING CLERK</t>
         </is>
       </c>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-      <c r="H60" s="17"/>
-      <c r="L60" s="17" t="inlineStr">
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="L60" t="inlineStr" s="153">
         <is>
           <t>PRESIDENT</t>
         </is>
       </c>
-      <c r="M60" s="17"/>
-      <c r="C60" s="14"/>
-      <c r="I60" s="17"/>
-      <c r="J60" s="17"/>
-      <c r="K60" s="17"/>
-      <c r="N60" s="17"/>
-      <c r="O60" s="17"/>
-    </row>
-    <row r="61" spans="2:40" ht="16.149999999999999" customHeight="1" ns2:dyDescent="0.25"/>
-    <row r="65" spans="29:49" ns2:dyDescent="0.25">
-      <c r="AN65"/>
-    </row>
-    <row r="66" spans="29:49" ns2:dyDescent="0.25">
-      <c r="AN66"/>
-    </row>
-    <row r="67" spans="29:49" ht="15" customHeight="1" ns2:dyDescent="0.25">
-      <c r="AN67"/>
-    </row>
-    <row r="68" spans="29:49" ht="16.899999999999999" customHeight="1" ns2:dyDescent="0.35">
+      <c r="M60" s="153"/>
+    </row>
+    <row ht="16.149999999999999" customHeight="1" r="61" spans="2:40" ns2:dyDescent="0.25"/>
+    <row r="65" spans="29:49" ns2:dyDescent="0.25"/>
+    <row r="66" spans="29:49" ns2:dyDescent="0.25"/>
+    <row ht="15" customHeight="1" r="67" spans="29:49" ns2:dyDescent="0.25"/>
+    <row ht="16.899999999999999" customHeight="1" r="68" spans="29:49" ns2:dyDescent="0.35">
       <c r="AC68" s="53"/>
       <c r="AD68" s="54"/>
       <c r="AE68" s="54"/>
@@ -9341,12 +8587,11 @@
       <c r="AK68" s="54"/>
       <c r="AL68" s="54"/>
       <c r="AM68" s="54"/>
-      <c r="AN68"/>
       <c r="AQ68" s="53"/>
       <c r="AR68" s="52"/>
       <c r="AS68" s="55"/>
     </row>
-    <row r="69" spans="29:49" ht="31.9" customHeight="1" ns2:dyDescent="0.25"/>
+    <row ht="31.9" customHeight="1" r="69" spans="29:49" ns2:dyDescent="0.25"/>
     <row r="71" spans="29:49" ns2:dyDescent="0.25">
       <c r="AU71" s="21"/>
       <c r="AV71" s="21"/>
@@ -9391,7 +8636,7 @@
       <c r="AQ82" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="21">
     <mergeCell ref="B43:N43"/>
     <mergeCell ref="B44:N44"/>
     <mergeCell ref="L60:M60"/>
@@ -9413,8 +8658,6 @@
     <mergeCell ref="AT18:AV18"/>
     <mergeCell ref="AO18:AQ18"/>
     <mergeCell ref="AZ18:BB18"/>
-    <mergeCell ref="B40:O40"/>
-    <mergeCell ref="B41:O41"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(export): fit four Main Office employees in management workbook
Insert a styled employee row in the Main Office template sheet and
shift the TOTAL, sign-off, overtime and journal rows down by one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/payroll/management-template.xlsx
+++ b/resources/payroll/management-template.xlsx
@@ -2155,7 +2155,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A3:DN72"/>
+  <dimension ref="A3:DN73"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" ns2:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -2899,333 +2899,439 @@
       <c r="DM12" s="1"/>
       <c r="DN12" s="1"/>
     </row>
-    <row r="13" spans="1:118" ns2:dyDescent="0.25">
+    <row r="13" spans="1:118" s="143" customFormat="1" ns2:dyDescent="0.25">
       <c r="A13" s="144"/>
-      <c r="B13" s="128"/>
-      <c r="C13" s="128"/>
-      <c r="D13" s="129"/>
-      <c r="E13" s="130"/>
-      <c r="F13" s="131"/>
-      <c r="G13" s="131"/>
-      <c r="H13" s="130"/>
-      <c r="I13" s="131"/>
-      <c r="J13" s="131"/>
-      <c r="K13" s="132"/>
-      <c r="L13" s="133"/>
-      <c r="M13" s="133"/>
-      <c r="N13" s="145"/>
-      <c r="O13" s="134"/>
-      <c r="P13" s="135"/>
-      <c r="Q13" s="129"/>
-      <c r="R13" s="131"/>
-      <c r="S13" s="136"/>
-      <c r="T13" s="131"/>
-      <c r="U13" s="131"/>
-      <c r="V13" s="131"/>
-      <c r="W13" s="132"/>
-      <c r="X13" s="132"/>
-      <c r="Y13" s="132"/>
-      <c r="Z13" s="146"/>
-      <c r="AA13" s="144"/>
-      <c r="AB13" s="134"/>
-      <c r="AC13" s="137"/>
-      <c r="AD13" s="130"/>
-      <c r="AE13" s="130"/>
-      <c r="AF13" s="130"/>
-      <c r="AG13" s="130"/>
-      <c r="AH13" s="130"/>
-      <c r="AI13" s="130"/>
-      <c r="AJ13" s="130"/>
-      <c r="AK13" s="138"/>
-      <c r="AL13" s="145"/>
-      <c r="AM13" s="134"/>
-      <c r="AN13" s="139"/>
-      <c r="AO13" s="140"/>
-      <c r="AP13" s="140"/>
-      <c r="AQ13" s="140"/>
-      <c r="AR13" s="140"/>
-      <c r="AS13" s="140"/>
-      <c r="AT13" s="140"/>
-      <c r="AU13" s="140"/>
-      <c r="AV13" s="140"/>
-      <c r="AW13" s="145"/>
-      <c r="AX13" s="141"/>
-      <c r="AY13" s="139"/>
-      <c r="AZ13" s="139"/>
-      <c r="BA13" s="140"/>
-      <c r="BB13" s="140"/>
-      <c r="BC13" s="139"/>
-      <c r="BD13" s="139"/>
-      <c r="BE13" s="139"/>
-      <c r="BF13" s="139"/>
-      <c r="BG13" s="142"/>
-      <c r="BH13" s="147"/>
-      <c r="BI13" s="146"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="15"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="120"/>
+      <c r="T13" s="17"/>
+      <c r="U13" s="17"/>
+      <c r="V13" s="17"/>
+      <c r="W13" s="18"/>
+      <c r="X13" s="18"/>
+      <c r="Y13" s="18"/>
+      <c r="Z13" s="1"/>
+      <c r="AA13" s="1"/>
+      <c r="AB13" s="14"/>
+      <c r="AC13" s="22"/>
+      <c r="AD13" s="34"/>
+      <c r="AE13" s="34"/>
+      <c r="AF13" s="34"/>
+      <c r="AG13" s="34"/>
+      <c r="AH13" s="34"/>
+      <c r="AI13" s="34"/>
+      <c r="AJ13" s="34"/>
+      <c r="AK13" s="25"/>
+      <c r="AL13" s="1"/>
+      <c r="AM13" s="14"/>
+      <c r="AN13" s="30"/>
+      <c r="AO13" s="26"/>
+      <c r="AP13" s="26"/>
+      <c r="AQ13" s="26"/>
+      <c r="AR13" s="26"/>
+      <c r="AS13" s="26"/>
+      <c r="AT13" s="26"/>
+      <c r="AU13" s="26"/>
+      <c r="AV13" s="26"/>
+      <c r="AW13" s="1"/>
+      <c r="AX13" s="35"/>
+      <c r="AY13" s="30"/>
+      <c r="AZ13" s="30"/>
+      <c r="BA13" s="26"/>
+      <c r="BB13" s="26"/>
+      <c r="BC13" s="30"/>
+      <c r="BD13" s="30"/>
+      <c r="BE13" s="30"/>
+      <c r="BF13" s="30"/>
+      <c r="BG13" s="27"/>
+      <c r="BH13" s="30"/>
+      <c r="BI13" s="1"/>
+      <c r="BJ13" s="1"/>
+      <c r="BK13" s="1"/>
+      <c r="BL13" s="1"/>
+      <c r="BM13" s="1"/>
+      <c r="BN13" s="1"/>
+      <c r="BO13" s="1"/>
+      <c r="BP13" s="1"/>
+      <c r="BQ13" s="1"/>
+      <c r="BR13" s="1"/>
+      <c r="BS13" s="1"/>
+      <c r="BT13" s="1"/>
+      <c r="BU13" s="1"/>
+      <c r="BV13" s="1"/>
+      <c r="BW13" s="1"/>
+      <c r="BX13" s="1"/>
+      <c r="BY13" s="1"/>
+      <c r="BZ13" s="1"/>
+      <c r="CA13" s="1"/>
+      <c r="CB13" s="1"/>
+      <c r="CC13" s="1"/>
+      <c r="CD13" s="1"/>
+      <c r="CE13" s="1"/>
+      <c r="CF13" s="1"/>
+      <c r="CG13" s="1"/>
+      <c r="CH13" s="1"/>
+      <c r="CI13" s="1"/>
+      <c r="CJ13" s="1"/>
+      <c r="CK13" s="1"/>
+      <c r="CL13" s="1"/>
+      <c r="CM13" s="1"/>
+      <c r="CN13" s="1"/>
+      <c r="CO13" s="1"/>
+      <c r="CP13" s="1"/>
+      <c r="CQ13" s="1"/>
+      <c r="CR13" s="1"/>
+      <c r="CS13" s="1"/>
+      <c r="CT13" s="1"/>
+      <c r="CU13" s="1"/>
+      <c r="CV13" s="1"/>
+      <c r="CW13" s="1"/>
+      <c r="CX13" s="1"/>
+      <c r="CY13" s="1"/>
+      <c r="CZ13" s="1"/>
+      <c r="DA13" s="1"/>
+      <c r="DB13" s="1"/>
+      <c r="DC13" s="1"/>
+      <c r="DD13" s="1"/>
+      <c r="DE13" s="1"/>
+      <c r="DF13" s="1"/>
+      <c r="DG13" s="1"/>
+      <c r="DH13" s="1"/>
+      <c r="DI13" s="1"/>
+      <c r="DJ13" s="1"/>
+      <c r="DK13" s="1"/>
+      <c r="DL13" s="1"/>
+      <c r="DM13" s="1"/>
+      <c r="DN13" s="1"/>
     </row>
     <row r="14" spans="1:118" ns2:dyDescent="0.25">
-      <c r="B14" s="158" t="inlineStr">
+      <c r="A14" s="144"/>
+      <c r="B14" s="128"/>
+      <c r="C14" s="128"/>
+      <c r="D14" s="129"/>
+      <c r="E14" s="130"/>
+      <c r="F14" s="131"/>
+      <c r="G14" s="131"/>
+      <c r="H14" s="130"/>
+      <c r="I14" s="131"/>
+      <c r="J14" s="131"/>
+      <c r="K14" s="132"/>
+      <c r="L14" s="133"/>
+      <c r="M14" s="133"/>
+      <c r="N14" s="145"/>
+      <c r="O14" s="134"/>
+      <c r="P14" s="135"/>
+      <c r="Q14" s="129"/>
+      <c r="R14" s="131"/>
+      <c r="S14" s="136"/>
+      <c r="T14" s="131"/>
+      <c r="U14" s="131"/>
+      <c r="V14" s="131"/>
+      <c r="W14" s="132"/>
+      <c r="X14" s="132"/>
+      <c r="Y14" s="132"/>
+      <c r="Z14" s="146"/>
+      <c r="AA14" s="144"/>
+      <c r="AB14" s="134"/>
+      <c r="AC14" s="137"/>
+      <c r="AD14" s="130"/>
+      <c r="AE14" s="130"/>
+      <c r="AF14" s="130"/>
+      <c r="AG14" s="130"/>
+      <c r="AH14" s="130"/>
+      <c r="AI14" s="130"/>
+      <c r="AJ14" s="130"/>
+      <c r="AK14" s="138"/>
+      <c r="AL14" s="145"/>
+      <c r="AM14" s="134"/>
+      <c r="AN14" s="139"/>
+      <c r="AO14" s="140"/>
+      <c r="AP14" s="140"/>
+      <c r="AQ14" s="140"/>
+      <c r="AR14" s="140"/>
+      <c r="AS14" s="140"/>
+      <c r="AT14" s="140"/>
+      <c r="AU14" s="140"/>
+      <c r="AV14" s="140"/>
+      <c r="AW14" s="145"/>
+      <c r="AX14" s="141"/>
+      <c r="AY14" s="139"/>
+      <c r="AZ14" s="139"/>
+      <c r="BA14" s="140"/>
+      <c r="BB14" s="140"/>
+      <c r="BC14" s="139"/>
+      <c r="BD14" s="139"/>
+      <c r="BE14" s="139"/>
+      <c r="BF14" s="139"/>
+      <c r="BG14" s="142"/>
+      <c r="BH14" s="147"/>
+      <c r="BI14" s="146"/>
+    </row>
+    <row r="15" spans="1:118" ns2:dyDescent="0.25">
+      <c r="B15" s="158" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="158"/>
-      <c r="D14" s="158"/>
-      <c r="E14" s="158"/>
-      <c r="F14" s="158"/>
-      <c r="G14" s="158"/>
-      <c r="H14" s="158"/>
-      <c r="I14" s="158"/>
-      <c r="J14" s="158"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="O14" s="158" t="inlineStr">
+      <c r="C15" s="158"/>
+      <c r="D15" s="158"/>
+      <c r="E15" s="158"/>
+      <c r="F15" s="158"/>
+      <c r="G15" s="158"/>
+      <c r="H15" s="158"/>
+      <c r="I15" s="158"/>
+      <c r="J15" s="158"/>
+      <c r="K15" s="36"/>
+      <c r="L15" s="36"/>
+      <c r="M15" s="36"/>
+      <c r="O15" s="158" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="P14" s="158"/>
-      <c r="Q14" s="158"/>
-      <c r="R14" s="158"/>
-      <c r="S14" s="158"/>
-      <c r="T14" s="158"/>
-      <c r="U14" s="158"/>
-      <c r="V14" s="158"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="119"/>
-      <c r="Y14" s="36"/>
-      <c r="AC14" s="37"/>
-      <c r="AD14" s="37"/>
-      <c r="AE14" s="37"/>
-      <c r="AF14" s="37"/>
-      <c r="AG14" s="37"/>
-      <c r="AH14" s="37"/>
-      <c r="AI14" s="37"/>
-      <c r="AJ14" s="37"/>
-      <c r="AK14" s="37"/>
-      <c r="AN14" s="37"/>
-      <c r="AO14" s="37"/>
-      <c r="AP14" s="37"/>
-      <c r="AQ14" s="37"/>
-      <c r="AR14" s="37"/>
-      <c r="AS14" s="37"/>
-      <c r="AT14" s="37"/>
-      <c r="AU14" s="37"/>
-      <c r="AV14" s="37"/>
-      <c r="AY14" s="37"/>
-      <c r="AZ14" s="37"/>
-      <c r="BA14" s="37"/>
-      <c r="BB14" s="37"/>
-      <c r="BC14" s="37"/>
-      <c r="BD14" s="37"/>
-      <c r="BE14" s="37"/>
-      <c r="BF14" s="37"/>
-      <c r="BG14" s="37"/>
-      <c r="BH14" s="37"/>
-    </row>
-    <row r="16" spans="1:118" ns2:dyDescent="0.25">
-      <c r="B16" s="1" t="inlineStr">
+      <c r="P15" s="158"/>
+      <c r="Q15" s="158"/>
+      <c r="R15" s="158"/>
+      <c r="S15" s="158"/>
+      <c r="T15" s="158"/>
+      <c r="U15" s="158"/>
+      <c r="V15" s="158"/>
+      <c r="W15" s="36"/>
+      <c r="X15" s="119"/>
+      <c r="Y15" s="36"/>
+      <c r="AC15" s="37"/>
+      <c r="AD15" s="37"/>
+      <c r="AE15" s="37"/>
+      <c r="AF15" s="37"/>
+      <c r="AG15" s="37"/>
+      <c r="AH15" s="37"/>
+      <c r="AI15" s="37"/>
+      <c r="AJ15" s="37"/>
+      <c r="AK15" s="37"/>
+      <c r="AN15" s="37"/>
+      <c r="AO15" s="37"/>
+      <c r="AP15" s="37"/>
+      <c r="AQ15" s="37"/>
+      <c r="AR15" s="37"/>
+      <c r="AS15" s="37"/>
+      <c r="AT15" s="37"/>
+      <c r="AU15" s="37"/>
+      <c r="AV15" s="37"/>
+      <c r="AY15" s="37"/>
+      <c r="AZ15" s="37"/>
+      <c r="BA15" s="37"/>
+      <c r="BB15" s="37"/>
+      <c r="BC15" s="37"/>
+      <c r="BD15" s="37"/>
+      <c r="BE15" s="37"/>
+      <c r="BF15" s="37"/>
+      <c r="BG15" s="37"/>
+      <c r="BH15" s="37"/>
+    </row>
+    <row r="17" spans="1:118" ns2:dyDescent="0.25">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Prepared by:</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Certified Correct:</t>
         </is>
       </c>
-      <c r="J16" s="1" t="inlineStr">
+      <c r="J17" s="1" t="inlineStr">
         <is>
           <t>Approved by:</t>
         </is>
       </c>
-      <c r="O16" s="1" t="inlineStr">
+      <c r="O17" s="1" t="inlineStr">
         <is>
           <t>Prepared by:</t>
         </is>
       </c>
-      <c r="Q16" s="1" t="inlineStr">
+      <c r="Q17" s="1" t="inlineStr">
         <is>
           <t>Certified Correct:</t>
         </is>
       </c>
-      <c r="V16" s="1" t="inlineStr">
+      <c r="V17" s="1" t="inlineStr">
         <is>
           <t>Approved by:</t>
         </is>
       </c>
     </row>
-    <row r="18" spans="2:60" ht="15.6" customHeight="1" ns2:dyDescent="0.25">
-      <c r="B18" s="39"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="K18" s="8"/>
-      <c r="O18" s="39"/>
-      <c r="Q18" s="160"/>
-      <c r="R18" s="160"/>
-      <c r="S18" s="160"/>
-      <c r="T18" s="9"/>
-      <c r="W18" s="8"/>
-      <c r="X18" s="8"/>
-      <c r="AN18" s="38"/>
-      <c r="AO18" s="38"/>
-    </row>
-    <row r="19" spans="2:60" ht="24" thickBot="1" ns2:dyDescent="0.3">
-      <c r="B19" s="10" t="inlineStr">
+    <row r="19" spans="2:60" ht="15.6" customHeight="1" ns2:dyDescent="0.25">
+      <c r="B19" s="39"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="K19" s="8"/>
+      <c r="O19" s="39"/>
+      <c r="Q19" s="160"/>
+      <c r="R19" s="160"/>
+      <c r="S19" s="160"/>
+      <c r="T19" s="9"/>
+      <c r="W19" s="8"/>
+      <c r="X19" s="8"/>
+      <c r="AN19" s="38"/>
+      <c r="AO19" s="38"/>
+    </row>
+    <row r="20" spans="2:60" ht="24" thickBot="1" ns2:dyDescent="0.3">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>PAYROLL OFFICER</t>
         </is>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>ACCOUNTING CLERK</t>
         </is>
       </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="K19" s="153" t="inlineStr">
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="K20" s="153" t="inlineStr">
         <is>
           <t>PRESIDENT</t>
         </is>
       </c>
-      <c r="L19" s="153"/>
-      <c r="O19" s="10" t="inlineStr">
+      <c r="L20" s="153"/>
+      <c r="O20" s="10" t="inlineStr">
         <is>
           <t>PAYROLL OFFICER</t>
         </is>
       </c>
-      <c r="Q19" s="159" t="inlineStr">
+      <c r="Q20" s="159" t="inlineStr">
         <is>
           <t>ACCOUNTING CLERK</t>
         </is>
       </c>
-      <c r="R19" s="159"/>
-      <c r="S19" s="159"/>
-      <c r="T19" s="4"/>
-      <c r="W19" s="153" t="inlineStr">
+      <c r="R20" s="159"/>
+      <c r="S20" s="159"/>
+      <c r="T20" s="4"/>
+      <c r="W20" s="153" t="inlineStr">
         <is>
           <t>PRESIDENT</t>
         </is>
       </c>
-      <c r="X19" s="153"/>
-      <c r="AM19" s="155" t="inlineStr">
+      <c r="X20" s="153"/>
+      <c r="AM20" s="155" t="inlineStr">
         <is>
           <t>OVERTIME PAY</t>
         </is>
       </c>
-      <c r="AN19" s="155"/>
-      <c r="AO19" s="155"/>
-      <c r="AR19" s="154" t="inlineStr">
+      <c r="AN20" s="155"/>
+      <c r="AO20" s="155"/>
+      <c r="AR20" s="154" t="inlineStr">
         <is>
           <t>1.3% OVERTIME</t>
         </is>
       </c>
-      <c r="AS19" s="154"/>
-      <c r="AT19" s="154"/>
-      <c r="AU19" s="57"/>
-      <c r="AV19" s="8"/>
-      <c r="AX19" s="155" t="inlineStr">
+      <c r="AS20" s="154"/>
+      <c r="AT20" s="154"/>
+      <c r="AU20" s="57"/>
+      <c r="AV20" s="8"/>
+      <c r="AX20" s="155" t="inlineStr">
         <is>
           <t>OVERTIME PAY</t>
         </is>
       </c>
-      <c r="AY19" s="155"/>
-      <c r="AZ19" s="155"/>
-      <c r="BC19" s="154" t="inlineStr">
+      <c r="AY20" s="155"/>
+      <c r="AZ20" s="155"/>
+      <c r="BC20" s="154" t="inlineStr">
         <is>
           <t>1.3% OVERTIME</t>
         </is>
       </c>
-      <c r="BD19" s="154"/>
-      <c r="BE19" s="154"/>
-      <c r="BF19" s="57"/>
-      <c r="BG19" s="8"/>
-      <c r="BH19" s="8"/>
-    </row>
-    <row r="20" spans="2:60" ht="32.25" thickTop="1" ns2:dyDescent="0.25">
-      <c r="AM20" s="40" t="inlineStr">
+      <c r="BD20" s="154"/>
+      <c r="BE20" s="154"/>
+      <c r="BF20" s="57"/>
+      <c r="BG20" s="8"/>
+      <c r="BH20" s="8"/>
+    </row>
+    <row r="21" spans="2:60" ht="32.25" thickTop="1" ns2:dyDescent="0.25">
+      <c r="AM21" s="40" t="inlineStr">
         <is>
           <t>EMPLOYEE NAME</t>
         </is>
       </c>
-      <c r="AN20" s="41" t="inlineStr">
+      <c r="AN21" s="41" t="inlineStr">
         <is>
           <t>NO OF HOURS</t>
         </is>
       </c>
-      <c r="AO20" s="41" t="inlineStr">
+      <c r="AO21" s="41" t="inlineStr">
         <is>
           <t>TOTAL OT PAY</t>
         </is>
       </c>
-      <c r="AR20" s="11" t="inlineStr">
+      <c r="AR21" s="11" t="inlineStr">
         <is>
           <t>EMPLOYEE NAME</t>
         </is>
       </c>
-      <c r="AS20" s="42" t="inlineStr">
+      <c r="AS21" s="42" t="inlineStr">
         <is>
           <t>NO OF HOURS</t>
         </is>
       </c>
-      <c r="AT20" s="42" t="inlineStr">
+      <c r="AT21" s="42" t="inlineStr">
         <is>
           <t>TOTAL OT PAY</t>
         </is>
       </c>
-      <c r="AX20" s="40" t="inlineStr">
+      <c r="AX21" s="40" t="inlineStr">
         <is>
           <t>EMPLOYEE NAME</t>
         </is>
       </c>
-      <c r="AY20" s="41" t="inlineStr">
+      <c r="AY21" s="41" t="inlineStr">
         <is>
           <t>NO OF HOURS</t>
         </is>
       </c>
-      <c r="AZ20" s="41" t="inlineStr">
+      <c r="AZ21" s="41" t="inlineStr">
         <is>
           <t>TOTAL OT PAY</t>
         </is>
       </c>
-      <c r="BC20" s="11" t="inlineStr">
+      <c r="BC21" s="11" t="inlineStr">
         <is>
           <t>EMPLOYEE NAME</t>
         </is>
       </c>
-      <c r="BD20" s="42" t="inlineStr">
+      <c r="BD21" s="42" t="inlineStr">
         <is>
           <t>NO OF HOURS</t>
         </is>
       </c>
-      <c r="BE20" s="42" t="inlineStr">
+      <c r="BE21" s="42" t="inlineStr">
         <is>
           <t>TOTAL OT PAY</t>
         </is>
       </c>
-      <c r="BH20" s="4"/>
-    </row>
-    <row r="21" spans="2:60" ns2:dyDescent="0.25">
-      <c r="M21" s="8"/>
-      <c r="AM21" s="14"/>
-      <c r="AN21" s="43"/>
-      <c r="AO21" s="44"/>
-      <c r="AR21" s="14"/>
-      <c r="AS21" s="45"/>
-      <c r="AT21" s="46"/>
-      <c r="AX21" s="14"/>
-      <c r="AY21" s="43"/>
-      <c r="AZ21" s="44"/>
-      <c r="BC21" s="14"/>
-      <c r="BD21" s="45"/>
-      <c r="BE21" s="46"/>
+      <c r="BH21" s="4"/>
     </row>
     <row r="22" spans="2:60" ns2:dyDescent="0.25">
+      <c r="M22" s="8"/>
       <c r="AM22" s="14"/>
       <c r="AN22" s="43"/>
       <c r="AO22" s="44"/>
@@ -3239,256 +3345,276 @@
       <c r="BD22" s="45"/>
       <c r="BE22" s="46"/>
     </row>
-    <row r="24" spans="2:60" ht="15.6" customHeight="1" ns2:dyDescent="0.25">
-      <c r="P24" s="1" t="inlineStr">
+    <row r="23" spans="2:60" ns2:dyDescent="0.25">
+      <c r="AM23" s="14"/>
+      <c r="AN23" s="43"/>
+      <c r="AO23" s="44"/>
+      <c r="AR23" s="14"/>
+      <c r="AS23" s="45"/>
+      <c r="AT23" s="46"/>
+      <c r="AX23" s="14"/>
+      <c r="AY23" s="43"/>
+      <c r="AZ23" s="44"/>
+      <c r="BC23" s="14"/>
+      <c r="BD23" s="45"/>
+      <c r="BE23" s="46"/>
+    </row>
+    <row r="24" spans="2:60">
+      <c r="AM24" s="14"/>
+      <c r="AN24" s="43"/>
+      <c r="AO24" s="44"/>
+      <c r="AR24" s="14"/>
+      <c r="AS24" s="45"/>
+      <c r="AT24" s="46"/>
+      <c r="AX24" s="14"/>
+      <c r="AY24" s="43"/>
+      <c r="AZ24" s="44"/>
+      <c r="BC24" s="14"/>
+      <c r="BD24" s="45"/>
+      <c r="BE24" s="46"/>
+    </row>
+    <row r="25" spans="2:60" ht="15.6" customHeight="1" ns2:dyDescent="0.25">
+      <c r="P25" s="1" t="inlineStr">
         <is>
           <t>Salaries and Wages</t>
         </is>
       </c>
-      <c r="R24" s="47"/>
-      <c r="X24" s="48"/>
-    </row>
-    <row r="25" spans="2:60" ht="16.149999999999999" customHeight="1" ns2:dyDescent="0.25">
-      <c r="L25" s="47"/>
-      <c r="P25" s="1" t="inlineStr">
+      <c r="R25" s="47"/>
+      <c r="X25" s="48"/>
+      <c r="AM25" s="14"/>
+      <c r="AN25" s="43"/>
+      <c r="AO25" s="44"/>
+      <c r="AR25" s="14"/>
+      <c r="AS25" s="45"/>
+      <c r="AT25" s="46"/>
+      <c r="AX25" s="14"/>
+      <c r="AY25" s="43"/>
+      <c r="AZ25" s="44"/>
+      <c r="BC25" s="14"/>
+      <c r="BD25" s="45"/>
+      <c r="BE25" s="46"/>
+    </row>
+    <row r="26" spans="2:60" ht="16.149999999999999" customHeight="1" ns2:dyDescent="0.25">
+      <c r="L26" s="47"/>
+      <c r="P26" s="1" t="inlineStr">
         <is>
           <t>    Wholding Tax Payable</t>
         </is>
       </c>
-      <c r="S25" s="5"/>
-      <c r="T25" s="5"/>
-    </row>
-    <row r="26" spans="2:60" ns2:dyDescent="0.25">
-      <c r="P26" s="1" t="inlineStr">
-        <is>
-          <t>     SSS Payable</t>
-        </is>
-      </c>
-      <c r="S26" s="48"/>
-      <c r="T26" s="48"/>
+      <c r="S26" s="5"/>
+      <c r="T26" s="5"/>
     </row>
     <row r="27" spans="2:60" ns2:dyDescent="0.25">
       <c r="P27" s="1" t="inlineStr">
         <is>
-          <t>     Phil Health Payable</t>
-        </is>
-      </c>
-      <c r="S27" s="21"/>
-      <c r="T27" s="21"/>
-      <c r="AM27" s="1" t="inlineStr">
-        <is>
-          <t>Prepared by:</t>
-        </is>
-      </c>
-      <c r="AP27" s="1" t="inlineStr">
-        <is>
-          <t>Certified Correct:</t>
-        </is>
-      </c>
-      <c r="AT27" s="49" t="inlineStr">
-        <is>
-          <t>Approved by:</t>
-        </is>
-      </c>
-      <c r="AX27" s="1" t="inlineStr">
-        <is>
-          <t>Prepared by:</t>
-        </is>
-      </c>
-      <c r="BA27" s="1" t="inlineStr">
-        <is>
-          <t>Certified Correct:</t>
-        </is>
-      </c>
-      <c r="BE27" s="49" t="inlineStr">
-        <is>
-          <t>Approved by:</t>
-        </is>
-      </c>
+          <t>     SSS Payable</t>
+        </is>
+      </c>
+      <c r="S27" s="48"/>
+      <c r="T27" s="48"/>
     </row>
     <row r="28" spans="2:60" ns2:dyDescent="0.25">
       <c r="P28" s="1" t="inlineStr">
         <is>
-          <t>     PAGIBIG Contribution</t>
-        </is>
-      </c>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
+          <t>     Phil Health Payable</t>
+        </is>
+      </c>
+      <c r="S28" s="21"/>
+      <c r="T28" s="21"/>
+      <c r="AM28" s="1" t="inlineStr">
+        <is>
+          <t>Prepared by:</t>
+        </is>
+      </c>
+      <c r="AP28" s="1" t="inlineStr">
+        <is>
+          <t>Certified Correct:</t>
+        </is>
+      </c>
+      <c r="AT28" s="49" t="inlineStr">
+        <is>
+          <t>Approved by:</t>
+        </is>
+      </c>
+      <c r="AX28" s="1" t="inlineStr">
+        <is>
+          <t>Prepared by:</t>
+        </is>
+      </c>
+      <c r="BA28" s="1" t="inlineStr">
+        <is>
+          <t>Certified Correct:</t>
+        </is>
+      </c>
+      <c r="BE28" s="49" t="inlineStr">
+        <is>
+          <t>Approved by:</t>
+        </is>
+      </c>
     </row>
     <row r="29" spans="2:60" ns2:dyDescent="0.25">
       <c r="P29" s="1" t="inlineStr">
         <is>
+          <t>     PAGIBIG Contribution</t>
+        </is>
+      </c>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+    </row>
+    <row r="30" spans="2:60" ns2:dyDescent="0.25">
+      <c r="P30" s="1" t="inlineStr">
+        <is>
           <t>     Loans Recievable - Long Term</t>
         </is>
       </c>
-      <c r="S29" s="48"/>
-      <c r="T29" s="5"/>
-      <c r="AM29" s="39"/>
-      <c r="AP29" s="39"/>
-      <c r="AQ29" s="8"/>
-      <c r="AU29" s="7"/>
-      <c r="AX29" s="39"/>
-      <c r="BA29" s="39"/>
-      <c r="BB29" s="8"/>
-      <c r="BF29" s="7"/>
-    </row>
-    <row r="30" spans="2:60" ns2:dyDescent="0.25">
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="P30" s="1" t="inlineStr">
+      <c r="S30" s="48"/>
+      <c r="T30" s="5"/>
+      <c r="AM30" s="39"/>
+      <c r="AP30" s="39"/>
+      <c r="AQ30" s="8"/>
+      <c r="AU30" s="7"/>
+      <c r="AX30" s="39"/>
+      <c r="BA30" s="39"/>
+      <c r="BB30" s="8"/>
+      <c r="BF30" s="7"/>
+    </row>
+    <row r="31" spans="2:60" ns2:dyDescent="0.25">
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="P31" s="1" t="inlineStr">
         <is>
           <t>     Interest income from  Loans</t>
         </is>
       </c>
-      <c r="S30" s="48"/>
-      <c r="T30" s="21"/>
-      <c r="U30" s="48"/>
-      <c r="AM30" s="10" t="inlineStr">
+      <c r="S31" s="48"/>
+      <c r="T31" s="21"/>
+      <c r="U31" s="48"/>
+      <c r="AM31" s="10" t="inlineStr">
         <is>
           <t>PAYROLL OFFICER</t>
         </is>
       </c>
-      <c r="AP30" s="10"/>
-      <c r="AQ30" s="4" t="inlineStr">
+      <c r="AP31" s="10"/>
+      <c r="AQ31" s="4" t="inlineStr">
         <is>
           <t>ACCOUNTING CLERK</t>
         </is>
       </c>
-      <c r="AR30" s="4"/>
-      <c r="AS30" s="10"/>
-      <c r="AT30" s="10"/>
-      <c r="AU30" s="10" t="inlineStr">
+      <c r="AR31" s="4"/>
+      <c r="AS31" s="10"/>
+      <c r="AT31" s="10"/>
+      <c r="AU31" s="10" t="inlineStr">
         <is>
           <t>PRESIDENT</t>
         </is>
       </c>
-      <c r="AX30" s="10" t="inlineStr">
+      <c r="AX31" s="10" t="inlineStr">
         <is>
           <t>PAYROLL OFFICER</t>
         </is>
       </c>
-      <c r="BA30" s="10"/>
-      <c r="BB30" s="4" t="inlineStr">
+      <c r="BA31" s="10"/>
+      <c r="BB31" s="4" t="inlineStr">
         <is>
           <t>ACCOUNTING CLERK</t>
         </is>
       </c>
-      <c r="BC30" s="4"/>
-      <c r="BD30" s="10"/>
-      <c r="BE30" s="10"/>
-      <c r="BF30" s="10" t="inlineStr">
+      <c r="BC31" s="4"/>
+      <c r="BD31" s="10"/>
+      <c r="BE31" s="10"/>
+      <c r="BF31" s="10" t="inlineStr">
         <is>
           <t>PRESIDENT</t>
         </is>
       </c>
-    </row>
-    <row r="31" spans="2:60" ns2:dyDescent="0.25">
-      <c r="P31" s="1" t="inlineStr">
-        <is>
-          <t>     Share Capital - Preferred</t>
-        </is>
-      </c>
-      <c r="S31" s="21"/>
-      <c r="T31" s="47"/>
     </row>
     <row r="32" spans="2:60" ns2:dyDescent="0.25">
       <c r="P32" s="1" t="inlineStr">
         <is>
+          <t>     Share Capital - Preferred</t>
+        </is>
+      </c>
+      <c r="S32" s="21"/>
+      <c r="T32" s="47"/>
+    </row>
+    <row r="33" spans="2:60" ns2:dyDescent="0.25">
+      <c r="P33" s="1" t="inlineStr">
+        <is>
           <t>     Rental Income</t>
         </is>
       </c>
-      <c r="S32" s="5"/>
-      <c r="T32" s="50"/>
-      <c r="V32" s="48"/>
-    </row>
-    <row r="33" spans="1:38" ns2:dyDescent="0.25">
-      <c r="B33" s="151"/>
-      <c r="C33" s="151"/>
-      <c r="D33" s="151"/>
-      <c r="E33" s="151"/>
-      <c r="F33" s="151"/>
-      <c r="G33" s="151"/>
-      <c r="H33" s="151"/>
-      <c r="I33" s="151"/>
-      <c r="J33" s="151"/>
-      <c r="K33" s="151"/>
-      <c r="L33" s="151"/>
-      <c r="M33" s="151"/>
-      <c r="N33" s="151"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1" t="inlineStr">
+      <c r="S33" s="5"/>
+      <c r="T33" s="50"/>
+      <c r="V33" s="48"/>
+    </row>
+    <row r="34" spans="1:38" ns2:dyDescent="0.25">
+      <c r="B34" s="151"/>
+      <c r="C34" s="151"/>
+      <c r="D34" s="151"/>
+      <c r="E34" s="151"/>
+      <c r="F34" s="151"/>
+      <c r="G34" s="151"/>
+      <c r="H34" s="151"/>
+      <c r="I34" s="151"/>
+      <c r="J34" s="151"/>
+      <c r="K34" s="151"/>
+      <c r="L34" s="151"/>
+      <c r="M34" s="151"/>
+      <c r="N34" s="151"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1" t="inlineStr">
         <is>
           <t>     Savings Deposit</t>
         </is>
       </c>
-      <c r="S33" s="21"/>
-      <c r="T33" s="48"/>
-    </row>
-    <row r="34" spans="1:38" ns2:dyDescent="0.25">
-      <c r="A34" s="10"/>
-      <c r="B34" s="152"/>
-      <c r="C34" s="152"/>
-      <c r="D34" s="152"/>
-      <c r="E34" s="152"/>
-      <c r="F34" s="152"/>
-      <c r="G34" s="152"/>
-      <c r="H34" s="152"/>
-      <c r="I34" s="152"/>
-      <c r="J34" s="152"/>
-      <c r="K34" s="152"/>
-      <c r="L34" s="152"/>
-      <c r="M34" s="152"/>
-      <c r="N34" s="152"/>
-      <c r="P34" s="1" t="inlineStr">
+      <c r="S34" s="21"/>
+      <c r="T34" s="48"/>
+    </row>
+    <row r="35" spans="1:38" ns2:dyDescent="0.25">
+      <c r="A35" s="10"/>
+      <c r="B35" s="152"/>
+      <c r="C35" s="152"/>
+      <c r="D35" s="152"/>
+      <c r="E35" s="152"/>
+      <c r="F35" s="152"/>
+      <c r="G35" s="152"/>
+      <c r="H35" s="152"/>
+      <c r="I35" s="152"/>
+      <c r="J35" s="152"/>
+      <c r="K35" s="152"/>
+      <c r="L35" s="152"/>
+      <c r="M35" s="152"/>
+      <c r="N35" s="152"/>
+      <c r="P35" s="1" t="inlineStr">
         <is>
           <t>     Employees' Benefit (13 Month Pay, Bonus Allowance Others)</t>
         </is>
       </c>
-      <c r="S34" s="21"/>
-      <c r="T34" s="21"/>
-    </row>
-    <row r="35" spans="1:38" ns2:dyDescent="0.25">
-      <c r="B35" s="39"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="113"/>
-      <c r="E35" s="113"/>
-      <c r="F35" s="113"/>
-      <c r="G35" s="113"/>
-      <c r="H35" s="113"/>
-      <c r="I35" s="113"/>
-      <c r="J35" s="113"/>
-      <c r="K35" s="39"/>
-      <c r="L35" s="113"/>
-      <c r="M35" s="113"/>
-      <c r="P35" s="1" t="inlineStr">
+      <c r="S35" s="21"/>
+      <c r="T35" s="21"/>
+    </row>
+    <row r="36" spans="1:38" ns2:dyDescent="0.25">
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="113"/>
+      <c r="E36" s="113"/>
+      <c r="F36" s="113"/>
+      <c r="G36" s="113"/>
+      <c r="H36" s="113"/>
+      <c r="I36" s="113"/>
+      <c r="J36" s="113"/>
+      <c r="K36" s="39"/>
+      <c r="L36" s="113"/>
+      <c r="M36" s="113"/>
+      <c r="P36" s="1" t="inlineStr">
         <is>
           <t>     Advances To Officers, Employees and Members</t>
         </is>
       </c>
-      <c r="S35" s="21"/>
-    </row>
-    <row r="36" spans="1:38" ns2:dyDescent="0.25">
-      <c r="B36" s="53"/>
-      <c r="C36" s="114"/>
-      <c r="D36" s="115"/>
-      <c r="E36" s="116"/>
-      <c r="F36" s="116"/>
-      <c r="G36" s="116"/>
-      <c r="H36" s="116"/>
-      <c r="I36" s="116"/>
-      <c r="J36" s="106"/>
-      <c r="K36" s="117"/>
-      <c r="L36" s="117"/>
-      <c r="M36" s="117"/>
-      <c r="P36" s="1" t="inlineStr">
-        <is>
-          <t>     Other Income</t>
-        </is>
-      </c>
-      <c r="S36" s="5"/>
+      <c r="S36" s="21"/>
     </row>
     <row r="37" spans="1:38" ns2:dyDescent="0.25">
       <c r="B37" s="53"/>
@@ -3505,148 +3631,162 @@
       <c r="M37" s="117"/>
       <c r="P37" s="1" t="inlineStr">
         <is>
+          <t>     Other Income</t>
+        </is>
+      </c>
+      <c r="S37" s="5"/>
+    </row>
+    <row r="38" spans="1:38" ns2:dyDescent="0.25">
+      <c r="B38" s="53"/>
+      <c r="C38" s="114"/>
+      <c r="D38" s="115"/>
+      <c r="E38" s="116"/>
+      <c r="F38" s="116"/>
+      <c r="G38" s="116"/>
+      <c r="H38" s="116"/>
+      <c r="I38" s="116"/>
+      <c r="J38" s="106"/>
+      <c r="K38" s="117"/>
+      <c r="L38" s="117"/>
+      <c r="M38" s="117"/>
+      <c r="P38" s="1" t="inlineStr">
+        <is>
           <t>     Cash in Bank</t>
         </is>
       </c>
-      <c r="S37" s="47"/>
-    </row>
-    <row r="38" spans="1:38" ns2:dyDescent="0.25">
-      <c r="B38" s="149"/>
-      <c r="C38" s="149"/>
-      <c r="D38" s="149"/>
-      <c r="E38" s="149"/>
-      <c r="F38" s="149"/>
-      <c r="G38" s="149"/>
-      <c r="H38" s="149"/>
-      <c r="I38" s="149"/>
-      <c r="J38" s="36"/>
-      <c r="K38" s="36"/>
-      <c r="L38" s="36"/>
-      <c r="M38" s="36"/>
-      <c r="R38" s="106"/>
-      <c r="S38" s="50"/>
-      <c r="T38" s="5"/>
-      <c r="AC38" s="5"/>
-      <c r="AF38" s="5"/>
-      <c r="AG38" s="50"/>
+      <c r="S38" s="47"/>
     </row>
     <row r="39" spans="1:38" ns2:dyDescent="0.25">
-      <c r="C39" s="118"/>
-      <c r="D39" s="118"/>
-      <c r="E39" s="118"/>
-      <c r="F39" s="118"/>
-      <c r="G39" s="118"/>
-      <c r="H39" s="118"/>
-      <c r="I39" s="118"/>
-      <c r="J39" s="118"/>
+      <c r="B39" s="149"/>
+      <c r="C39" s="149"/>
+      <c r="D39" s="149"/>
+      <c r="E39" s="149"/>
+      <c r="F39" s="149"/>
+      <c r="G39" s="149"/>
+      <c r="H39" s="149"/>
+      <c r="I39" s="149"/>
+      <c r="J39" s="36"/>
       <c r="K39" s="36"/>
       <c r="L39" s="36"/>
       <c r="M39" s="36"/>
-      <c r="N39" s="37"/>
-      <c r="T39" s="48"/>
+      <c r="R39" s="106"/>
+      <c r="S39" s="50"/>
+      <c r="T39" s="5"/>
+      <c r="AC39" s="5"/>
+      <c r="AF39" s="5"/>
+      <c r="AG39" s="50"/>
     </row>
     <row r="40" spans="1:38" ns2:dyDescent="0.25">
-      <c r="T40" s="21"/>
-    </row>
-    <row r="41"/>
-    <row r="42" spans="1:38" ns2:dyDescent="0.25">
-      <c r="AB42" s="5"/>
-      <c r="AC42" s="5"/>
-      <c r="AG42" s="5"/>
-    </row>
-    <row r="43"/>
-    <row r="44" spans="1:38" ns2:dyDescent="0.25">
-      <c r="B44" s="39"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="9"/>
-      <c r="L44" s="7"/>
-      <c r="AC44" s="5"/>
-    </row>
+      <c r="C40" s="118"/>
+      <c r="D40" s="118"/>
+      <c r="E40" s="118"/>
+      <c r="F40" s="118"/>
+      <c r="G40" s="118"/>
+      <c r="H40" s="118"/>
+      <c r="I40" s="118"/>
+      <c r="J40" s="118"/>
+      <c r="K40" s="36"/>
+      <c r="L40" s="36"/>
+      <c r="M40" s="36"/>
+      <c r="N40" s="37"/>
+      <c r="T40" s="48"/>
+    </row>
+    <row r="41" spans="1:38" ns2:dyDescent="0.25">
+      <c r="T41" s="21"/>
+    </row>
+    <row r="42"/>
+    <row r="43" spans="1:38" ns2:dyDescent="0.25">
+      <c r="AB43" s="5"/>
+      <c r="AC43" s="5"/>
+      <c r="AG43" s="5"/>
+    </row>
+    <row r="44"/>
     <row r="45" spans="1:38" ns2:dyDescent="0.25">
-      <c r="B45" s="10"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="L45" s="112"/>
-      <c r="AC45" s="6"/>
-      <c r="AD45" s="6"/>
-      <c r="AE45" s="6"/>
-      <c r="AF45" s="51"/>
-      <c r="AG45" s="52"/>
-      <c r="AH45" s="50"/>
-      <c r="AI45" s="50"/>
+      <c r="B45" s="39"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="L45" s="7"/>
+      <c r="AC45" s="5"/>
     </row>
     <row r="46" spans="1:38" ns2:dyDescent="0.25">
-      <c r="AC46" s="5"/>
-      <c r="AD46" s="5"/>
-      <c r="AE46" s="5"/>
-      <c r="AF46" s="5"/>
-      <c r="AG46" s="5"/>
-      <c r="AH46" s="5"/>
-      <c r="AI46" s="5"/>
-      <c r="AJ46" s="5"/>
-      <c r="AK46" s="5"/>
-    </row>
-    <row r="47"/>
-    <row ht="15.6" customHeight="1" r="48" spans="1:38" ns2:dyDescent="0.25">
-      <c r="AL48" s="38"/>
-    </row>
-    <row ht="16.149999999999999" customHeight="1" r="49" spans="28:47" ns2:dyDescent="0.25">
+      <c r="B46" s="10"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="L46" s="112"/>
+      <c r="AC46" s="6"/>
+      <c r="AD46" s="6"/>
+      <c r="AE46" s="6"/>
+      <c r="AF46" s="51"/>
+      <c r="AG46" s="52"/>
+      <c r="AH46" s="50"/>
+      <c r="AI46" s="50"/>
+    </row>
+    <row r="47" spans="1:38" ns2:dyDescent="0.25">
+      <c r="AC47" s="5"/>
+      <c r="AD47" s="5"/>
+      <c r="AE47" s="5"/>
+      <c r="AF47" s="5"/>
+      <c r="AG47" s="5"/>
+      <c r="AH47" s="5"/>
+      <c r="AI47" s="5"/>
+      <c r="AJ47" s="5"/>
+      <c r="AK47" s="5"/>
+    </row>
+    <row r="48"/>
+    <row ht="15.6" customHeight="1" r="49" spans="1:38" ns2:dyDescent="0.25">
       <c r="AL49" s="38"/>
     </row>
-    <row r="50"/>
-    <row ht="16.149999999999999" customHeight="1" r="51" spans="28:47" ns2:dyDescent="0.25"/>
-    <row r="52"/>
+    <row ht="16.149999999999999" customHeight="1" r="50" spans="28:47" ns2:dyDescent="0.25">
+      <c r="AL50" s="38"/>
+    </row>
+    <row r="51"/>
+    <row ht="16.149999999999999" customHeight="1" r="52" spans="28:47" ns2:dyDescent="0.25"/>
     <row r="53"/>
     <row r="54"/>
-    <row r="55" spans="28:47" ns2:dyDescent="0.25"/>
+    <row r="55"/>
     <row r="56" spans="28:47" ns2:dyDescent="0.25"/>
-    <row ht="15" customHeight="1" r="57" spans="28:47" ns2:dyDescent="0.25"/>
-    <row ht="16.899999999999999" customHeight="1" r="58" spans="28:47" ns2:dyDescent="0.35">
-      <c r="AB58" s="53"/>
-      <c r="AC58" s="54"/>
-      <c r="AD58" s="54"/>
-      <c r="AE58" s="54"/>
-      <c r="AF58" s="54"/>
-      <c r="AG58" s="54"/>
-      <c r="AH58" s="54"/>
-      <c r="AI58" s="54"/>
-      <c r="AJ58" s="54"/>
-      <c r="AK58" s="54"/>
-      <c r="AO58" s="53"/>
-      <c r="AP58" s="52"/>
-      <c r="AQ58" s="55"/>
-    </row>
-    <row ht="31.9" customHeight="1" r="59" spans="28:47" ns2:dyDescent="0.25"/>
-    <row r="60"/>
-    <row r="61" spans="28:47" ns2:dyDescent="0.25">
-      <c r="AS61" s="21"/>
-      <c r="AT61" s="21"/>
-      <c r="AU61" s="5"/>
-    </row>
+    <row r="57" spans="28:47" ns2:dyDescent="0.25"/>
+    <row ht="15" customHeight="1" r="58" spans="28:47" ns2:dyDescent="0.25"/>
+    <row ht="16.899999999999999" customHeight="1" r="59" spans="28:47" ns2:dyDescent="0.35">
+      <c r="AB59" s="53"/>
+      <c r="AC59" s="54"/>
+      <c r="AD59" s="54"/>
+      <c r="AE59" s="54"/>
+      <c r="AF59" s="54"/>
+      <c r="AG59" s="54"/>
+      <c r="AH59" s="54"/>
+      <c r="AI59" s="54"/>
+      <c r="AJ59" s="54"/>
+      <c r="AK59" s="54"/>
+      <c r="AO59" s="53"/>
+      <c r="AP59" s="52"/>
+      <c r="AQ59" s="55"/>
+    </row>
+    <row ht="31.9" customHeight="1" r="60" spans="28:47" ns2:dyDescent="0.25"/>
+    <row r="61"/>
     <row r="62" spans="28:47" ns2:dyDescent="0.25">
-      <c r="AR62" s="56"/>
       <c r="AS62" s="21"/>
       <c r="AT62" s="21"/>
       <c r="AU62" s="5"/>
     </row>
     <row r="63" spans="28:47" ns2:dyDescent="0.25">
+      <c r="AR63" s="56"/>
       <c r="AS63" s="21"/>
       <c r="AT63" s="21"/>
       <c r="AU63" s="5"/>
     </row>
     <row r="64" spans="28:47" ns2:dyDescent="0.25">
-      <c r="AR64" s="56"/>
       <c r="AS64" s="21"/>
       <c r="AT64" s="21"/>
       <c r="AU64" s="5"/>
     </row>
-    <row r="65" spans="41:47" ns2:dyDescent="0.25">
+    <row r="65" spans="28:47" ns2:dyDescent="0.25">
       <c r="AR65" s="56"/>
       <c r="AS65" s="21"/>
       <c r="AT65" s="21"/>
@@ -3664,8 +3804,14 @@
       <c r="AT67" s="21"/>
       <c r="AU67" s="5"/>
     </row>
-    <row r="72" spans="41:47" ns2:dyDescent="0.25">
-      <c r="AO72" s="21"/>
+    <row r="68" spans="41:47" ns2:dyDescent="0.25">
+      <c r="AR68" s="56"/>
+      <c r="AS68" s="21"/>
+      <c r="AT68" s="21"/>
+      <c r="AU68" s="5"/>
+    </row>
+    <row r="73" spans="41:47" ns2:dyDescent="0.25">
+      <c r="AO73" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -3675,37 +3821,37 @@
     <mergeCell ref="B9:M9"/>
     <mergeCell ref="O9:Y9"/>
     <mergeCell ref="AX9:BH9"/>
-    <mergeCell ref="AM19:AO19"/>
-    <mergeCell ref="AR19:AT19"/>
+    <mergeCell ref="AM20:AO20"/>
+    <mergeCell ref="AR20:AT20"/>
     <mergeCell ref="AM9:AV9"/>
+    <mergeCell ref="Q20:S20"/>
     <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="W19:X19"/>
-    <mergeCell ref="AX19:AZ19"/>
-    <mergeCell ref="BC19:BE19"/>
-    <mergeCell ref="O14:V14"/>
+    <mergeCell ref="W20:X20"/>
+    <mergeCell ref="AX20:AZ20"/>
+    <mergeCell ref="BC20:BE20"/>
+    <mergeCell ref="O15:V15"/>
+    <mergeCell ref="B35:N35"/>
+    <mergeCell ref="B39:I39"/>
     <mergeCell ref="B34:N34"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="B15:J15"/>
   </mergeCells>
-  <conditionalFormatting sqref="AB11 AB13">
+  <conditionalFormatting sqref="AB11 AB14">
     <cfRule type="duplicateValues" dxfId="5" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB12">
+  <conditionalFormatting sqref="AB12:AB13">
     <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM11 AM13">
+  <conditionalFormatting sqref="AM11 AM14">
     <cfRule type="duplicateValues" dxfId="3" priority="41"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM12">
+  <conditionalFormatting sqref="AM12:AM13">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AX11 AX13">
+  <conditionalFormatting sqref="AX11 AX14">
     <cfRule type="duplicateValues" dxfId="1" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AX12">
+  <conditionalFormatting sqref="AX12:AX13">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>